<commit_message>
new file:   INSTALL.md new file:   Map1 (7).xlsx 	modified:   README.md 	new file:   TRA_OUT_815_GL040868.csv 	modified:   config/flows.yaml 	new file:   data/README.md 	new file:   data/inbound/archive/.gitkeep
</commit_message>
<xml_diff>
--- a/examples/mapping ROLLS SSW outgoing.xlsx
+++ b/examples/mapping ROLLS SSW outgoing.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29825"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29905"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://totalworkplace-my.sharepoint.com/personal/leander_fransoo_external_totalenergies_com/Documents/Documents/LOT 1/integratie rolls/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="487" documentId="8_{95FF6B5B-68D7-48DE-B19B-5019895BC047}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{07658655-1CC2-493D-B425-C29251882717}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{8D70C991-53B2-434E-BAD4-D59E1149158C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-30852" yWindow="-132" windowWidth="30984" windowHeight="16824" firstSheet="7" xr2:uid="{F5622C39-BDEB-4266-9322-5FC9E204C153}"/>
+    <workbookView xWindow="-30852" yWindow="-132" windowWidth="30984" windowHeight="16824" xr2:uid="{F5622C39-BDEB-4266-9322-5FC9E204C153}"/>
   </bookViews>
   <sheets>
     <sheet name="CSV to XML" sheetId="1" r:id="rId1"/>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="373" uniqueCount="266">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="432" uniqueCount="291">
   <si>
     <t>Kolom nr</t>
   </si>
@@ -63,55 +63,52 @@
     <t>status</t>
   </si>
   <si>
-    <t>Kolom1</t>
-  </si>
-  <si>
-    <t>PldaSswDeclaration/typeDeclaration</t>
+    <t>Transform</t>
+  </si>
+  <si>
+    <t>/PldaSswDeclaration/typeDeclaration</t>
   </si>
   <si>
     <t>Vaste Tekst: PD</t>
   </si>
   <si>
-    <t>CSV to XML</t>
-  </si>
-  <si>
-    <t>PldaSswDeclaration/version</t>
+    <t>/PldaSswDeclaration/version</t>
   </si>
   <si>
     <t>Vaste Tekst: 1.0</t>
   </si>
   <si>
-    <t>PldaSswDeclaration/dateCreation</t>
+    <t>/PldaSswDeclaration/dateCreation</t>
   </si>
   <si>
     <t>T000580</t>
   </si>
   <si>
-    <t>PldaSswDeclaration/timeCreation</t>
+    <t>/PldaSswDeclaration/timeCreation</t>
   </si>
   <si>
     <t>T003941</t>
   </si>
   <si>
-    <t>PldaSswDeclaration/CustomsStreamliner/company</t>
+    <t>/PldaSswDeclaration/CustomsStreamliner/company</t>
   </si>
   <si>
     <t>Vaste tekst: TE</t>
   </si>
   <si>
-    <t>PldaSswDeclaration/MessageBody/SADDossier/GoodsDeclaration/type</t>
-  </si>
-  <si>
-    <t>O</t>
-  </si>
-  <si>
-    <t>PldaSswDeclaration/MessageBody/SADDossier/GoodsDeclaration/linkId</t>
+    <t>/PldaSswDeclaration/MessageBody/SADDossier/GoodsDeclaration/type</t>
+  </si>
+  <si>
+    <t>Vaste tekst: O</t>
+  </si>
+  <si>
+    <t>/PldaSswDeclaration/MessageBody/SADDossier/GoodsDeclaration/linkId</t>
   </si>
   <si>
     <t>T003422</t>
   </si>
   <si>
-    <t>PldaSswDeclaration/MessageBody/SADDossier/GoodsDeclaration/overview1</t>
+    <t>/PldaSswDeclaration/MessageBody/SADDossier/GoodsDeclaration/overview1</t>
   </si>
   <si>
     <t>T004093</t>
@@ -120,13 +117,19 @@
     <t>Type order van ROLLS</t>
   </si>
   <si>
-    <t>PldaSswDeclaration/MessageBody/SADDossier/GoodsDeclaration/Outbound/departedTime</t>
-  </si>
-  <si>
-    <t>PldaSswDeclaration/MessageBody/SADDossier/GoodsDeclaration/Outbound/departedDate</t>
-  </si>
-  <si>
-    <t>PldaSswDeclaration/MessageBody/SADDossier/GoodsDeclaration/Outbound/destinationCountry</t>
+    <t>/PldaSswDeclaration/MessageBody/SADDossier/GoodsDeclaration/Outbound/departedTime</t>
+  </si>
+  <si>
+    <t>not found in example</t>
+  </si>
+  <si>
+    <t>skip</t>
+  </si>
+  <si>
+    <t>/PldaSswDeclaration/MessageBody/SADDossier/GoodsDeclaration/Outbound/departedDate</t>
+  </si>
+  <si>
+    <t>/PldaSswDeclaration/MessageBody/SADDossier/GoodsDeclaration/Outbound/destinationCountry</t>
   </si>
   <si>
     <t>T004478</t>
@@ -135,34 +138,40 @@
     <t>eerste 2 karaketers gebruiken</t>
   </si>
   <si>
-    <t>/PldaSswDeclaration/MessageBody/SADDossier/GoodsDeclaration/outbound/ConsigneeEMCS/Operator/operatorName</t>
+    <t>/PldaSswDeclaration/MessageBody/SADDossier/GoodsDeclaration/Outbound/ConsigneeEMCS/Operator/OperatorAddress/country</t>
+  </si>
+  <si>
+    <t>reuse of column 11</t>
+  </si>
+  <si>
+    <t>/PldaSswDeclaration/MessageBody/SADDossier/GoodsDeclaration/Outbound/ConsigneeEMCS/Operator/operatorName</t>
   </si>
   <si>
     <t>T000244</t>
   </si>
   <si>
-    <t>/PldaSswDeclaration/MessageBody/SADDossier/GoodsDeclaration/outbound/ConsigneeEMCS/Operator/OperatorAddress/postalCode</t>
+    <t>/PldaSswDeclaration/MessageBody/SADDossier/GoodsDeclaration/Outbound/ConsigneeEMCS/Operator/OperatorAddress/postalCode</t>
   </si>
   <si>
     <t>T000254</t>
   </si>
   <si>
-    <t>/PldaSswDeclaration/MessageBody/SADDossier/GoodsDeclaration/outbound/ConsigneeEMCS/Operator/OperatorAddress/streetAndNumber1</t>
+    <t>/PldaSswDeclaration/MessageBody/SADDossier/GoodsDeclaration/Outbound/ConsigneeEMCS/Operator/OperatorAddress/streetAndNumber1</t>
   </si>
   <si>
     <t>T000247 + ‘ ‘ + T000249</t>
   </si>
   <si>
-    <t>/PldaSswDeclaration/MessageBody/SADDossier/GoodsDeclaration/outbound/ConsigneeEMCS/Operator/OperatorAddress/city</t>
+    <t>/PldaSswDeclaration/MessageBody/SADDossier/GoodsDeclaration/Outbound/ConsigneeEMCS/Operator/OperatorAddress/city</t>
   </si>
   <si>
     <t>T000251</t>
   </si>
   <si>
-    <t>/PldaSswDeclaration/MessageBody/SADDossier/GoodsDeclaration/outbound/ConsigneeEMCS/Operator/exciseNumber</t>
-  </si>
-  <si>
-    <t>/PldaSswDeclaration/MessageBody/SADDossier/GoodsDeclaration/outbound/ConsigneeEMCS/erpId</t>
+    <t>/PldaSswDeclaration/MessageBody/SADDossier/GoodsDeclaration/Outbound/ConsigneeEMCS/Operator/exciseNumber</t>
+  </si>
+  <si>
+    <t>/PldaSswDeclaration/MessageBody/SADDossier/GoodsDeclaration/Outbound/ConsigneeEMCS/erpId</t>
   </si>
   <si>
     <t>/PldaSswDeclaration/MessageBody/SADDossier/GoodsDeclaration/dossierDate</t>
@@ -201,10 +210,13 @@
     <t>T004614_1+T004614_2+T004614_3</t>
   </si>
   <si>
+    <t>first_27</t>
+  </si>
+  <si>
     <t>/PldaSswDeclaration/MessageBody/SADDossier/GoodsDeclaration/TransportMeans/dispatchCountry</t>
   </si>
   <si>
-    <t>Vaste Tekst:BE</t>
+    <t>Vaste Tekst: BE. Not found in example</t>
   </si>
   <si>
     <t>/PldaSswDeclaration/MessageBody/SADDossier/GoodsDeclaration/TransportMeans/transportType</t>
@@ -213,13 +225,19 @@
     <t>T004615_1</t>
   </si>
   <si>
+    <t>Xpath not found?</t>
+  </si>
+  <si>
     <t>/PldaSswDeclaration/MessageBody/SADDossier/GoodsDeclaration/TransportMeans/departureNationality</t>
   </si>
   <si>
+    <t>Vaste Tekst: BE</t>
+  </si>
+  <si>
     <t>/PldaSswDeclaration/MessageBody/SADDossier/GoodsDeclaration/businessUnit</t>
   </si>
   <si>
-    <t>Vaste Tekst:TERA</t>
+    <t>Vaste Tekst: TERA</t>
   </si>
   <si>
     <t>/PldaSswDeclaration/MessageBody/SADDossier/GoodsItem/sequence</t>
@@ -228,7 +246,10 @@
     <t>/PldaSswDeclaration/MessageBody/SADDossier/GoodsItem/Outbound/stockType</t>
   </si>
   <si>
-    <t>Vaste Tekst:EXCISE</t>
+    <t>Vaste Tekst: EXCISE</t>
+  </si>
+  <si>
+    <t>Vaste Tekst: TE_NOSTOCK</t>
   </si>
   <si>
     <t>/PldaSswDeclaration/MessageBody/SADDossier/GoodsItem/Product/code</t>
@@ -246,7 +267,7 @@
     <t>/PldaSswDeclaration/MessageBody/SADDossier/GoodsItem/Product/CommodityImport/typeDeclaration</t>
   </si>
   <si>
-    <t>Vaste Tekst:PI</t>
+    <t>Vaste Tekst: PI. Not found in example</t>
   </si>
   <si>
     <t>/PldaSswDeclaration/MessageBody/SADDossier/GoodsItem/Product/CommodityImport/commodityCode</t>
@@ -261,18 +282,21 @@
     <t>/PldaSswDeclaration/MessageBody/SADDossier/GoodsItem/Product/stockLevel</t>
   </si>
   <si>
-    <t>Vaste Tekst:LTR</t>
+    <t>Vaste Tekst: LTR</t>
   </si>
   <si>
     <t>/PldaSswDeclaration/MessageBody/SADDossier/GoodsItem/Product/declareLevel</t>
   </si>
   <si>
-    <t>Vaste Tekst:KGM</t>
+    <t>Vaste Tekst: KGM</t>
   </si>
   <si>
     <t>/PldaSswDeclaration/MessageBody/SADDossier/GoodsItem/Product/exciseProductCode</t>
   </si>
   <si>
+    <t>not found in example &amp; ook double? zie lijn 118</t>
+  </si>
+  <si>
     <t>/PldaSswDeclaration/MessageBody/SADDossier/GoodsItem/Product/CommercialDescription/commercialDescriptionLanguage</t>
   </si>
   <si>
@@ -288,25 +312,25 @@
     <t>T004668</t>
   </si>
   <si>
-    <t>/PldaSswDeclaration/MessageBody/SADDossier/GoodsItem/Product/goodsDescription</t>
-  </si>
-  <si>
-    <t>/PldaSswDeclaration/MessageBody/SADDossier/GoodsItem/Product/originCountry</t>
-  </si>
-  <si>
-    <t>/PldaSswDeclaration/MessageBody/SADDossier/GoodsItem/Product/netMass</t>
+    <t>/PldaSswDeclaration/MessageBody/SADDossier/GoodsItem/goodsDescription</t>
+  </si>
+  <si>
+    <t>/PldaSswDeclaration/MessageBody/SADDossier/GoodsItem/originCountry</t>
+  </si>
+  <si>
+    <t>/PldaSswDeclaration/MessageBody/SADDossier/GoodsItem/netMass</t>
   </si>
   <si>
     <t>T001634</t>
   </si>
   <si>
-    <t>/PldaSswDeclaration/MessageBody/SADDossier/GoodsItem/Product/grosMass</t>
+    <t>/PldaSswDeclaration/MessageBody/SADDossier/GoodsItem/grossMass</t>
   </si>
   <si>
     <t>T001633</t>
   </si>
   <si>
-    <t>/PldaSswDeclaration/MessageBody/SADDossier/GoodsItem/Product/stockAmount</t>
+    <t>/PldaSswDeclaration/MessageBody/SADDossier/GoodsItem/stockAmount</t>
   </si>
   <si>
     <t>T002727</t>
@@ -315,21 +339,18 @@
     <t>/PldaSswDeclaration/MessageBody/SADDossier/GoodsItem/Product/alcoholicStrength</t>
   </si>
   <si>
-    <t>/PldaSswDeclaration/MessageBody/SADDossier/GoodsItem/Product/Packaging/marksNumber</t>
+    <t>/PldaSswDeclaration/MessageBody/SADDossier/GoodsItem/Packaging/marksNumber</t>
   </si>
   <si>
     <t>Vaste Tekst: Deellading 1</t>
   </si>
   <si>
-    <t>/PldaSswDeclaration/MessageBody/SADDossier/GoodsItem/Product/packageType</t>
+    <t>/PldaSswDeclaration/MessageBody/SADDossier/GoodsItem/Packaging/packageType</t>
   </si>
   <si>
     <t>T001808</t>
   </si>
   <si>
-    <t>skip</t>
-  </si>
-  <si>
     <t>T000003</t>
   </si>
   <si>
@@ -354,7 +375,7 @@
     <t>T000014</t>
   </si>
   <si>
-    <t>SADDossier/GoodsDeclaration/DeliveryPlaceTrader/erpId</t>
+    <t>/PldaSswDeclaration/MessageBody/SADDossier/GoodsDeclaration/DeliveryPlaceTrader/erpId</t>
   </si>
   <si>
     <t>T000044</t>
@@ -363,82 +384,91 @@
     <t>T000083</t>
   </si>
   <si>
-    <t>SADDossier/GoodsDeclaration/Outbound/ConsigneeEMCS/Operator/language</t>
+    <t>/PldaSswDeclaration/MessageBody/SADDossier/GoodsDeclaration/DeliveryPlaceTrader/Operator/OperatorAddress/country</t>
+  </si>
+  <si>
+    <t>reuse of column 50</t>
+  </si>
+  <si>
+    <t>first_2</t>
+  </si>
+  <si>
+    <t>/PldaSswDeclaration/MessageBody/SADDossier/GoodsDeclaration/Outbound/ConsigneeEMCS/Operator/language</t>
   </si>
   <si>
     <t>T000245</t>
   </si>
   <si>
-    <t>SADDossier/GoodsDeclaration/Inbound/Consignor/Operator/operatorName</t>
+    <t>/PldaSswDeclaration/MessageBody/SADDossier/GoodsDeclaration/Inbound/Consignor/Operator/operatorName</t>
   </si>
   <si>
     <t>T000287</t>
   </si>
   <si>
-    <t>SADDossier/GoodsDeclaration/Inbound/Consignor/Operator/language</t>
+    <t>/PldaSswDeclaration/MessageBody/SADDossier/GoodsDeclaration/Inbound/Consignor/Operator/language</t>
   </si>
   <si>
     <t>T000288</t>
   </si>
   <si>
-    <t>SADDossier/GoodsDeclaration/Inbound/Consignor/Operator/OperatorAddress/streetAndNumber1</t>
+    <t>/PldaSswDeclaration/MessageBody/SADDossier/GoodsDeclaration/Inbound/Consignor/Operator/OperatorAddress/streetAndNumber1</t>
   </si>
   <si>
     <t>T000290+T004508</t>
   </si>
   <si>
-    <t>SADDossier/GoodsDeclaration/Inbound/Consignor/Operator/OperatorAddress/city</t>
+    <t>/PldaSswDeclaration/MessageBody/SADDossier/GoodsDeclaration/Inbound/Consignor/Operator/OperatorAddress/city</t>
   </si>
   <si>
     <t>T000292</t>
   </si>
   <si>
-    <t>SADDossier/GoodsDeclaration/Inbound/Consignor/Operator/OperatorAddress/postalCode</t>
+    <t>/PldaSswDeclaration/MessageBody/SADDossier/GoodsDeclaration/Inbound/Consignor/Operator/OperatorAddress/postalCode</t>
   </si>
   <si>
     <t>T000295</t>
   </si>
   <si>
-    <t>SADDossier/GoodsDeclaration/DeliveryPlaceTrader/Operator/operatorName</t>
+    <t>/PldaSswDeclaration/MessageBody/SADDossier/GoodsDeclaration/DeliveryPlaceTrader/Operator/operatorName</t>
   </si>
   <si>
     <t>T000390</t>
   </si>
   <si>
-    <t>SADDossier/GoodsDeclaration/DeliveryPlaceTrader/Operator/language</t>
+    <t>/PldaSswDeclaration/MessageBody/SADDossier/GoodsDeclaration/DeliveryPlaceTrader/Operator/language</t>
   </si>
   <si>
     <t>T000391</t>
   </si>
   <si>
-    <t>SADDossier/GoodsDeclaration/DeliveryPlaceTrader/Operator/OperatorAddress/streetAndNumber1</t>
+    <t>excisenumber &amp; exciseoffice mankeren</t>
+  </si>
+  <si>
+    <t>/PldaSswDeclaration/MessageBody/SADDossier/GoodsDeclaration/DeliveryPlaceTrader/Operator/OperatorAddress/streetAndNumber1</t>
   </si>
   <si>
     <t>T000393+T004696</t>
   </si>
   <si>
-    <t>SADDossier/GoodsDeclaration/DeliveryPlaceTrader/Operator/OperatorAddress/city</t>
+    <t>/PldaSswDeclaration/MessageBody/SADDossier/GoodsDeclaration/DeliveryPlaceTrader/Operator/OperatorAddress/city</t>
   </si>
   <si>
     <t>T000395</t>
   </si>
   <si>
-    <t>SADDossier/GoodsDeclaration/DeliveryPlaceTrader/Operator/OperatorAddress/postalCode</t>
+    <t>/PldaSswDeclaration/MessageBody/SADDossier/GoodsDeclaration/DeliveryPlaceTrader/Operator/OperatorAddress/postalCode</t>
   </si>
   <si>
     <t>T000398</t>
   </si>
   <si>
-    <t>SADDossier/GoodsDeclaration/overview1</t>
-  </si>
-  <si>
     <t>T000999</t>
   </si>
   <si>
     <t>indien value=="week" of "maand" dan kopiëren naar SADDossier/GoodsDeclaration/additionalScenarioSmartDeclare</t>
   </si>
   <si>
-    <t>PldaSswDeclaration/MessageBody/SADDossier/GoodsItem/linkId</t>
+    <t>/PldaSswDeclaration/MessageBody/SADDossier/GoodsItem/linkId</t>
   </si>
   <si>
     <t>T001379</t>
@@ -468,43 +498,55 @@
     <t>T004470</t>
   </si>
   <si>
-    <t>SADDossier/GoodsDeclaration/Inbound/Consignor/erpId</t>
+    <t>/PldaSswDeclaration/MessageBody/SADDossier/GoodsDeclaration/Inbound/Consignor/erpId</t>
   </si>
   <si>
     <t>T004485</t>
   </si>
   <si>
-    <t>SADDossier/GoodsDeclaration/DispatchTrader/erpId</t>
+    <t>/PldaSswDeclaration/MessageBody/SADDossier/GoodsDeclaration/Inbound/Consignor/Operator/OperatorAddress/country</t>
+  </si>
+  <si>
+    <t>reuse of column 64</t>
+  </si>
+  <si>
+    <t>/PldaSswDeclaration/MessageBody/SADDossier/GoodsDeclaration/DispatchTrader/erpId</t>
   </si>
   <si>
     <t>T004490</t>
   </si>
   <si>
-    <t>SADDossier/GoodsDeclaration/DispatchTrader/Operator/operatorName</t>
+    <t>/PldaSswDeclaration/MessageBody/SADDossier/GoodsDeclaration/DispatchTrader/Operator/OperatorAddress/country</t>
+  </si>
+  <si>
+    <t>reuse of column 65</t>
+  </si>
+  <si>
+    <t>/PldaSswDeclaration/MessageBody/SADDossier/GoodsDeclaration/DispatchTrader/Operator/operatorName</t>
   </si>
   <si>
     <t>T004493</t>
   </si>
   <si>
-    <t>SADDossier/GoodsDeclaration/DispatchTrader/Operator/language</t>
+    <t>/PldaSswDeclaration/MessageBody/SADDossier/GoodsDeclaration/DispatchTrader/Operator/language</t>
   </si>
   <si>
     <t>T004494</t>
   </si>
   <si>
-    <t>SADDossier/GoodsDeclaration/DispatchTrader/Operator/OperatorAddress/streetAndNumber1</t>
+    <t>/PldaSswDeclaration/MessageBody/SADDossier/GoodsDeclaration/DispatchTrader/Operator/OperatorAddress/streetAndNumber1</t>
   </si>
   <si>
     <t>T004496+T004498</t>
   </si>
   <si>
-    <t>SADDossier/GoodsDeclaration/DispatchTrader/Operator/OperatorAddress/city</t>
+    <t>/PldaSswDeclaration/MessageBody/SADDossier/GoodsDeclaration/DispatchTrader/Operator/OperatorAddress/city</t>
   </si>
   <si>
     <t>T004500</t>
   </si>
   <si>
-    <t>SADDossier/GoodsDeclaration/DispatchTrader/Operator/OperatorAddress/postalCode</t>
+    <t>/PldaSswDeclaration/MessageBody/SADDossier/GoodsDeclaration/DispatchTrader/Operator/OperatorAddress/postalCode</t>
   </si>
   <si>
     <t>T004504</t>
@@ -513,79 +555,91 @@
     <t>T004506</t>
   </si>
   <si>
-    <t>SADDossier/GoodsDeclaration/FirstTransporterTrader/erpId</t>
+    <t>/PldaSswDeclaration/MessageBody/SADDossier/GoodsDeclaration/FirstTransporterTrader/erpId</t>
   </si>
   <si>
     <t>T004514</t>
   </si>
   <si>
-    <t>SADDossier/GoodsDeclaration/FirstTransporterTrader/Operator/operatorName</t>
+    <t>/PldaSswDeclaration/MessageBody/SADDossier/GoodsDeclaration/FirstTransporterTrader/Operator/OperatorAddress/country</t>
+  </si>
+  <si>
+    <t>reuse of column 72</t>
+  </si>
+  <si>
+    <t>/PldaSswDeclaration/MessageBody/SADDossier/GoodsDeclaration/FirstTransporterTrader/Operator/operatorName</t>
   </si>
   <si>
     <t>T004516</t>
   </si>
   <si>
-    <t>SADDossier/GoodsDeclaration/FirstTransporterTrader/Operator/language</t>
+    <t>/PldaSswDeclaration/MessageBody/SADDossier/GoodsDeclaration/FirstTransporterTrader/Operator/language</t>
   </si>
   <si>
     <t>T004517</t>
   </si>
   <si>
-    <t>SADDossier/GoodsDeclaration/FirstTransporterTrader/Operator/OperatorAddress/streetAndNumber1</t>
+    <t>/PldaSswDeclaration/MessageBody/SADDossier/GoodsDeclaration/FirstTransporterTrader/Operator/OperatorAddress/streetAndNumber1</t>
   </si>
   <si>
     <t>T004519+T004521</t>
   </si>
   <si>
-    <t>SADDossier/GoodsDeclaration/FirstTransporterTrader/Operator/OperatorAddress/city</t>
+    <t>/PldaSswDeclaration/MessageBody/SADDossier/GoodsDeclaration/FirstTransporterTrader/Operator/OperatorAddress/city</t>
   </si>
   <si>
     <t>T004523</t>
   </si>
   <si>
-    <t>SADDossier/GoodsDeclaration/FirstTransporterTrader/Operator/OperatorAddress/postalCode</t>
+    <t>/PldaSswDeclaration/MessageBody/SADDossier/GoodsDeclaration/FirstTransporterTrader/Operator/OperatorAddress/postalCode</t>
   </si>
   <si>
     <t>T004527</t>
   </si>
   <si>
-    <t>SADDossier/GoodsDeclaration/TransportArrangerTrader/erpId</t>
+    <t>/PldaSswDeclaration/MessageBody/SADDossier/GoodsDeclaration/TransportArrangerTrader/erpId</t>
   </si>
   <si>
     <t>T004552</t>
   </si>
   <si>
-    <t>SADDossier/GoodsDeclaration/TransportArrangerTrader/Operator/operatorName</t>
+    <t>/PldaSswDeclaration/MessageBody/SADDossier/GoodsDeclaration/TransportArrangerTrader/Operator/OperatorAddress/country</t>
+  </si>
+  <si>
+    <t>reuse of column 78</t>
+  </si>
+  <si>
+    <t>/PldaSswDeclaration/MessageBody/SADDossier/GoodsDeclaration/TransportArrangerTrader/Operator/operatorName</t>
   </si>
   <si>
     <t>T004554</t>
   </si>
   <si>
-    <t>SADDossier/GoodsDeclaration/TransportArrangerTrader/Operator/language</t>
+    <t>/PldaSswDeclaration/MessageBody/SADDossier/GoodsDeclaration/TransportArrangerTrader/Operator/language</t>
   </si>
   <si>
     <t>T004555</t>
   </si>
   <si>
-    <t>SADDossier/GoodsDeclaration/TransportArrangerTrader/Operator/OperatorAddress/streetAndNumber1</t>
+    <t>/PldaSswDeclaration/MessageBody/SADDossier/GoodsDeclaration/TransportArrangerTrader/Operator/OperatorAddress/streetAndNumber1</t>
   </si>
   <si>
     <t>T004557+T004559</t>
   </si>
   <si>
-    <t>SADDossier/GoodsDeclaration/TransportArrangerTrader/Operator/OperatorAddress/city</t>
+    <t>/PldaSswDeclaration/MessageBody/SADDossier/GoodsDeclaration/TransportArrangerTrader/Operator/OperatorAddress/city</t>
   </si>
   <si>
     <t>T004561</t>
   </si>
   <si>
-    <t>SADDossier/GoodsDeclaration/TransportArrangerTrader/Operator/OperatorAddress/postalCode</t>
+    <t>/PldaSswDeclaration/MessageBody/SADDossier/GoodsDeclaration/TransportArrangerTrader/Operator/OperatorAddress/postalCode</t>
   </si>
   <si>
     <t>T004565</t>
   </si>
   <si>
-    <t>PldaSswDeclaration/MessageBody/SADDossier/GoodsDeclaration/overview2</t>
+    <t>/PldaSswDeclaration/MessageBody/SADDossier/GoodsDeclaration/overview2</t>
   </si>
   <si>
     <t>T004605</t>
@@ -594,13 +648,13 @@
     <t>`</t>
   </si>
   <si>
-    <t>SADDossier/GoodsDeclaration/Customs/exitOffice</t>
+    <t>/PldaSswDeclaration/MessageBody/SADDossier/GoodsDeclaration/Customs/exitOffice</t>
   </si>
   <si>
     <t>T004606</t>
   </si>
   <si>
-    <t>SADDossier/GoodsDeclaration/destinationType</t>
+    <t>/PldaSswDeclaration/MessageBody/SADDossier/GoodsDeclaration/destinationType</t>
   </si>
   <si>
     <t>T004608</t>
@@ -612,22 +666,22 @@
     <t>T004615_3</t>
   </si>
   <si>
-    <t>SADDossier/GoodsItem/ProducedDocument/Document/documentReference</t>
+    <t>/PldaSswDeclaration/MessageBody/SADDossier/GoodsItem/ProducedDocument/Document/documentReference</t>
   </si>
   <si>
     <t>T004618</t>
   </si>
   <si>
-    <t>SADDossier/GoodsItem/ProducedDocument/Document/emcsDocumentType</t>
+    <t>/PldaSswDeclaration/MessageBody/SADDossier/GoodsItem/ProducedDocument/Document/emcsDocumentType</t>
   </si>
   <si>
     <t>T004619</t>
   </si>
   <si>
-    <t>SADDossier/GoodsItem/ProducedDocument/Document/documentReferenceLanguage</t>
-  </si>
-  <si>
-    <t>SADDossier/GoodsDeclaration/TransportMeans/transportArrangment</t>
+    <t>/PldaSswDeclaration/MessageBody/SADDossier/GoodsItem/ProducedDocument/Document/documentReferenceLanguage</t>
+  </si>
+  <si>
+    <t>/PldaSswDeclaration/MessageBody/SADDossier/GoodsDeclaration/TransportMeans/transportArrangment</t>
   </si>
   <si>
     <t>T004625</t>
@@ -636,18 +690,12 @@
     <t>T004637</t>
   </si>
   <si>
-    <t>SADDossier/GoodsDeclaration/guarantorType</t>
+    <t>/PldaSswDeclaration/MessageBody/SADDossier/GoodsDeclaration/guarantorType</t>
   </si>
   <si>
     <t>T004638</t>
   </si>
   <si>
-    <t>SADDossier/GoodsItem/Product/exciseProductCode</t>
-  </si>
-  <si>
-    <t>SADDossier/GoodsItem/Product/code</t>
-  </si>
-  <si>
     <t>T004732</t>
   </si>
   <si>
@@ -801,10 +849,7 @@
     <t>Echte errorcode van EMCS</t>
   </si>
   <si>
-    <t>porthus stuurt dat de aangifte tot bij accijnzen is, nuttig om te weten tot waar bericht geraakt is</t>
-  </si>
-  <si>
-    <t>mapping nog te doen</t>
+    <t>is eigenlijk de aangifte zelf zoals in eerste sheet besproken, door SSW gewrapt in een EMCS formaat</t>
   </si>
   <si>
     <t>IE917</t>
@@ -828,9 +873,6 @@
     <t>EmcsSswArc/MessageBody/ie:IE704/ie:Body/ie:GenericRefusalMessage/ie:XmlError/ie:ie:ErrorLocation</t>
   </si>
   <si>
-    <t>Interfacing voor printopdracht van de declaratie vanuit ROLLS</t>
-  </si>
-  <si>
     <t>Intefacing voor foutmeldingen die vanuit stream zelf komen</t>
   </si>
   <si>
@@ -844,6 +886,39 @@
   </si>
   <si>
     <t>inhoudelijke transformaties gebeuren aan ROLLS kant</t>
+  </si>
+  <si>
+    <t>files (csv, xml, ...) moeten kunnen gefilterd worden op basis van naam</t>
+  </si>
+  <si>
+    <t>uitgaande declaratie</t>
+  </si>
+  <si>
+    <t>ie code</t>
+  </si>
+  <si>
+    <t>...</t>
+  </si>
+  <si>
+    <t>country voor operatoadress blokken afleiden uit 2eerste letters van gemapt veld uit csv</t>
+  </si>
+  <si>
+    <t>004478</t>
+  </si>
+  <si>
+    <t>004485</t>
+  </si>
+  <si>
+    <t>000044</t>
+  </si>
+  <si>
+    <t>004490</t>
+  </si>
+  <si>
+    <t>004514</t>
+  </si>
+  <si>
+    <t>004552</t>
   </si>
 </sst>
 </file>
@@ -953,7 +1028,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -975,6 +1050,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1135,7 +1216,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -1200,12 +1281,39 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="25">
+  <dxfs count="26">
     <dxf>
       <fill>
         <patternFill>
@@ -1465,6 +1573,13 @@
         </patternFill>
       </fill>
     </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -1479,15 +1594,15 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{D1007908-1428-46E5-B098-6287B5968C59}" name="Tabel1" displayName="Tabel1" ref="A1:F114" totalsRowShown="0" headerRowDxfId="18" headerRowBorderDxfId="16" tableBorderDxfId="17">
-  <autoFilter ref="A1:F114" xr:uid="{D1007908-1428-46E5-B098-6287B5968C59}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{D1007908-1428-46E5-B098-6287B5968C59}" name="Tabel1" displayName="Tabel1" ref="A1:F120" totalsRowShown="0" headerRowDxfId="18" headerRowBorderDxfId="16" tableBorderDxfId="17">
+  <autoFilter ref="A1:F120" xr:uid="{D1007908-1428-46E5-B098-6287B5968C59}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{AF48FF7C-1D1F-4ACF-8CC6-21402F1FCBFA}" name="Kolom nr" dataDxfId="15"/>
     <tableColumn id="2" xr3:uid="{56F2045E-3A52-41E1-8D01-629A0A10A63E}" name="Stream" dataDxfId="14"/>
     <tableColumn id="3" xr3:uid="{25248A49-0F74-4B1D-A7B2-DD89013C7126}" name="ROLLS Code"/>
     <tableColumn id="4" xr3:uid="{7EBD70C2-1BE3-4920-9F26-7AC8AAF0098B}" name="Opmerkingen"/>
     <tableColumn id="5" xr3:uid="{A82BAD71-3BF5-4993-BBA9-41C2EE7298FA}" name="status"/>
-    <tableColumn id="6" xr3:uid="{23B7B542-C044-4D1D-8E67-61DF0587A67A}" name="Kolom1"/>
+    <tableColumn id="6" xr3:uid="{23B7B542-C044-4D1D-8E67-61DF0587A67A}" name="Transform"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1824,7 +1939,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B52D4C27-6A8A-4E18-83AA-FB7C8AEF036F}">
-  <dimension ref="A1:F142"/>
+  <dimension ref="A1:F148"/>
   <sheetFormatPr defaultRowHeight="15.95"/>
   <cols>
     <col min="1" max="1" width="13.140625" customWidth="1"/>
@@ -1834,7 +1949,7 @@
     <col min="6" max="6" width="103.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="16.5" thickBot="1">
+    <row r="1" spans="1:6" ht="15.75">
       <c r="A1" s="10" t="s">
         <v>0</v>
       </c>
@@ -1865,20 +1980,18 @@
       <c r="D2" s="13" t="s">
         <v>7</v>
       </c>
-      <c r="F2" s="28" t="s">
-        <v>8</v>
-      </c>
+      <c r="F2" s="28"/>
     </row>
     <row r="3" spans="1:6" ht="15.75">
       <c r="A3" s="9">
         <v>1</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C3" s="12"/>
       <c r="D3" s="13" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="16.5" thickBot="1">
@@ -1886,10 +1999,10 @@
         <v>2</v>
       </c>
       <c r="B4" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>11</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="16.5" thickBot="1">
@@ -1897,10 +2010,10 @@
         <v>3</v>
       </c>
       <c r="B5" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C5" s="2" t="s">
         <v>13</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="15.75">
@@ -1908,70 +2021,77 @@
         <v>4</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C6" s="12"/>
       <c r="D6" s="13" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" ht="16.5" thickBot="1">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="15.75">
       <c r="A7" s="9">
         <v>5</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C7" s="12"/>
       <c r="D7" s="13" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" ht="16.5" thickBot="1">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="15.75">
       <c r="A8" s="9">
         <v>6</v>
       </c>
       <c r="B8" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C8" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="C8" s="2" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" ht="16.5" thickBot="1">
+    </row>
+    <row r="9" spans="1:6" ht="15.75">
       <c r="A9" s="9">
         <v>7</v>
       </c>
       <c r="B9" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="C9" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="D9" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="D9" s="14" t="s">
+    </row>
+    <row r="10" spans="1:6" ht="15.75">
+      <c r="A10" s="37">
+        <v>8</v>
+      </c>
+      <c r="B10" s="46" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" ht="16.5" thickBot="1">
-      <c r="A10" s="9">
-        <v>8</v>
-      </c>
-      <c r="B10" s="4" t="s">
+      <c r="C10" s="39" t="s">
+        <v>13</v>
+      </c>
+      <c r="D10" s="28" t="s">
         <v>24</v>
       </c>
-      <c r="C10" s="2" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" ht="16.5" thickBot="1">
+      <c r="E10" s="28"/>
+      <c r="F10" s="28" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="15.75">
       <c r="A11" s="9">
         <v>9</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="15.75">
@@ -1979,1279 +2099,1444 @@
         <v>10</v>
       </c>
       <c r="B12" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="D12" s="14" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" s="28" customFormat="1" ht="15.75">
+      <c r="A13" s="37">
+        <v>10</v>
+      </c>
+      <c r="B13" s="38" t="s">
+        <v>30</v>
+      </c>
+      <c r="C13" s="39" t="s">
+        <v>28</v>
+      </c>
+      <c r="D13" s="24" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" ht="15.75">
+      <c r="A14" s="9">
+        <v>11</v>
+      </c>
+      <c r="B14" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="C14" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="D14" s="14"/>
+    </row>
+    <row r="15" spans="1:6" ht="15.75">
+      <c r="A15" s="9">
+        <v>12</v>
+      </c>
+      <c r="B15" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="C15" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="D15" s="14"/>
+    </row>
+    <row r="16" spans="1:6" ht="15.75">
+      <c r="A16" s="9">
+        <v>13</v>
+      </c>
+      <c r="B16" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="C16" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="D16" s="14"/>
+    </row>
+    <row r="17" spans="1:6" ht="16.5" thickBot="1">
+      <c r="A17" s="9">
+        <v>14</v>
+      </c>
+      <c r="B17" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="D17" s="14"/>
+    </row>
+    <row r="18" spans="1:6" ht="16.5" thickBot="1">
+      <c r="A18" s="9">
+        <v>15</v>
+      </c>
+      <c r="B18" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="C18" t="s">
+        <v>28</v>
+      </c>
+      <c r="D18" s="14"/>
+    </row>
+    <row r="19" spans="1:6" ht="16.5" thickBot="1">
+      <c r="A19" s="9">
+        <v>16</v>
+      </c>
+      <c r="B19" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="C19" t="s">
+        <v>28</v>
+      </c>
+      <c r="D19" s="14"/>
+    </row>
+    <row r="20" spans="1:6" ht="16.5" thickBot="1">
+      <c r="A20" s="9">
+        <v>17</v>
+      </c>
+      <c r="B20" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D20" s="14"/>
+    </row>
+    <row r="21" spans="1:6" ht="15.75">
+      <c r="A21" s="9">
+        <v>18</v>
+      </c>
+      <c r="B21" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="D21" s="14"/>
+    </row>
+    <row r="22" spans="1:6" ht="16.5" thickBot="1">
+      <c r="A22" s="9">
+        <v>19</v>
+      </c>
+      <c r="B22" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="C22" s="6"/>
+      <c r="D22" s="43" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" ht="16.5" thickBot="1">
+      <c r="A23" s="9">
+        <v>20</v>
+      </c>
+      <c r="B23" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="C23" s="16" t="s">
+        <v>48</v>
+      </c>
+      <c r="D23" s="15"/>
+    </row>
+    <row r="24" spans="1:6" ht="16.5" thickBot="1">
+      <c r="A24" s="9">
+        <v>21</v>
+      </c>
+      <c r="B24" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="C24" s="16" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" s="35" customFormat="1" ht="15.75">
+      <c r="A25" s="32">
+        <v>22</v>
+      </c>
+      <c r="B25" s="33" t="s">
+        <v>50</v>
+      </c>
+      <c r="C25" s="33"/>
+      <c r="D25" s="34" t="s">
+        <v>51</v>
+      </c>
+      <c r="F25" s="35" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" ht="15.75">
+      <c r="A26" s="9">
+        <v>23</v>
+      </c>
+      <c r="B26" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="C26" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="F26" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" ht="16.5" thickBot="1">
+      <c r="A27" s="37">
+        <v>24</v>
+      </c>
+      <c r="B27" s="41" t="s">
+        <v>55</v>
+      </c>
+      <c r="C27" s="42"/>
+      <c r="D27" s="24" t="s">
+        <v>56</v>
+      </c>
+      <c r="E27" s="28"/>
+      <c r="F27" s="28" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" s="28" customFormat="1" ht="15.75">
+      <c r="A28" s="37">
+        <v>25</v>
+      </c>
+      <c r="B28" s="28" t="s">
+        <v>57</v>
+      </c>
+      <c r="C28" s="42" t="s">
+        <v>58</v>
+      </c>
+      <c r="D28" s="28" t="s">
+        <v>59</v>
+      </c>
+      <c r="F28" s="28" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" ht="16.5" thickBot="1">
+      <c r="A29" s="9">
         <v>26</v>
       </c>
-      <c r="C12" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="D12" s="14" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" ht="15.75">
-      <c r="A13" s="9">
-        <v>11</v>
-      </c>
-      <c r="B13" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="C13" s="8" t="s">
-        <v>30</v>
-      </c>
-      <c r="D13" s="14"/>
-    </row>
-    <row r="14" spans="1:6" ht="16.5" thickBot="1">
-      <c r="A14" s="9">
-        <v>12</v>
-      </c>
-      <c r="B14" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="C14" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="D14" s="14"/>
-    </row>
-    <row r="15" spans="1:6" ht="16.5" thickBot="1">
-      <c r="A15" s="9">
-        <v>13</v>
-      </c>
-      <c r="B15" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="C15" s="8" t="s">
-        <v>34</v>
-      </c>
-      <c r="D15" s="14"/>
-    </row>
-    <row r="16" spans="1:6" ht="16.5" thickBot="1">
-      <c r="A16" s="9">
-        <v>14</v>
-      </c>
-      <c r="B16" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="D16" s="14"/>
-    </row>
-    <row r="17" spans="1:4" ht="16.5" thickBot="1">
-      <c r="A17" s="9">
-        <v>15</v>
-      </c>
-      <c r="B17" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="C17" t="s">
-        <v>27</v>
-      </c>
-      <c r="D17" s="14"/>
-    </row>
-    <row r="18" spans="1:4" ht="16.5" thickBot="1">
-      <c r="A18" s="9">
-        <v>16</v>
-      </c>
-      <c r="B18" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="C18" t="s">
-        <v>27</v>
-      </c>
-      <c r="D18" s="14"/>
-    </row>
-    <row r="19" spans="1:4" ht="16.5" thickBot="1">
-      <c r="A19" s="9">
-        <v>17</v>
-      </c>
-      <c r="B19" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="C19" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="D19" s="14"/>
-    </row>
-    <row r="20" spans="1:4" ht="15.75">
-      <c r="A20" s="9">
-        <v>18</v>
-      </c>
-      <c r="B20" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="C20" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="D20" s="14"/>
-    </row>
-    <row r="21" spans="1:4" ht="16.5" thickBot="1">
-      <c r="A21" s="9">
-        <v>19</v>
-      </c>
-      <c r="B21" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="C21" s="6"/>
-      <c r="D21" s="32" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" ht="16.5" thickBot="1">
-      <c r="A22" s="9">
-        <v>20</v>
-      </c>
-      <c r="B22" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="C22" s="16" t="s">
-        <v>45</v>
-      </c>
-      <c r="D22" s="15"/>
-    </row>
-    <row r="23" spans="1:4" ht="16.5" thickBot="1">
-      <c r="A23" s="9">
-        <v>21</v>
-      </c>
-      <c r="B23" s="6" t="s">
-        <v>46</v>
-      </c>
-      <c r="C23" s="16" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" ht="15.75">
-      <c r="A24" s="9">
-        <v>22</v>
-      </c>
-      <c r="B24" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="C24" s="6"/>
-      <c r="D24" s="14" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" ht="15.75">
-      <c r="A25" s="9">
-        <v>23</v>
-      </c>
-      <c r="B25" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="C25" s="6" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" ht="16.5" thickBot="1">
-      <c r="A26" s="9">
-        <v>24</v>
-      </c>
-      <c r="B26" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="C26" s="6"/>
-      <c r="D26" s="14" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" ht="15.75">
-      <c r="A27" s="9">
-        <v>25</v>
-      </c>
-      <c r="B27" t="s">
-        <v>53</v>
-      </c>
-      <c r="C27" s="6" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" ht="16.5" thickBot="1">
-      <c r="A28" s="9">
-        <v>26</v>
-      </c>
-      <c r="B28" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="C28" s="6"/>
-      <c r="D28" s="14" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" ht="16.5" thickBot="1">
-      <c r="A29" s="9">
-        <v>27</v>
-      </c>
       <c r="B29" s="5" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="C29" s="6"/>
       <c r="D29" s="14" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4" ht="16.5" thickBot="1">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" ht="16.5" thickBot="1">
       <c r="A30" s="9">
+        <v>27</v>
+      </c>
+      <c r="B30" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="C30" s="6"/>
+      <c r="D30" s="14" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" ht="16.5" thickBot="1">
+      <c r="A31" s="9">
         <v>28</v>
       </c>
-      <c r="B30" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="C30" s="6"/>
-      <c r="D30" s="14">
+      <c r="B31" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="C31" s="6"/>
+      <c r="D31" s="14">
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:4" ht="16.5" thickBot="1">
-      <c r="A31" s="9">
+    <row r="32" spans="1:6" ht="16.5" thickBot="1">
+      <c r="A32" s="9">
         <v>29</v>
       </c>
-      <c r="B31" s="5" t="s">
-        <v>59</v>
-      </c>
-      <c r="C31" s="6"/>
-      <c r="D31" s="14" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4" ht="15.75">
-      <c r="A32" s="9">
+      <c r="B32" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="C32" s="6"/>
+      <c r="D32" s="14" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" ht="15.75">
+      <c r="A33" s="9">
         <v>30</v>
       </c>
-      <c r="B32" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="C32" s="6"/>
-      <c r="D32" s="32" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4" ht="15.75">
-      <c r="A33" s="9">
+      <c r="B33" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="C33" s="6"/>
+      <c r="D33" s="43" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" ht="15.75">
+      <c r="A34" s="9">
         <v>31</v>
       </c>
-      <c r="B33" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="C33" s="28" t="s">
-        <v>62</v>
-      </c>
-      <c r="D33" s="14"/>
-    </row>
-    <row r="34" spans="1:4" ht="16.5" thickBot="1">
-      <c r="A34" s="9">
+      <c r="B34" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="C34" s="30" t="s">
+        <v>69</v>
+      </c>
+      <c r="D34" s="14"/>
+    </row>
+    <row r="35" spans="1:6" ht="16.5" thickBot="1">
+      <c r="A35" s="9">
         <v>32</v>
       </c>
-      <c r="B34" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="C34" s="6" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4" ht="16.5" thickBot="1">
-      <c r="A35" s="9">
+      <c r="B35" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="C35" s="6" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" ht="16.5" thickBot="1">
+      <c r="A36" s="37">
         <v>33</v>
       </c>
-      <c r="B35" s="5" t="s">
-        <v>65</v>
-      </c>
-      <c r="C35" s="15"/>
-      <c r="D35" s="14" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="36" spans="1:4" ht="16.5" thickBot="1">
-      <c r="A36" s="9">
+      <c r="B36" s="41" t="s">
+        <v>72</v>
+      </c>
+      <c r="C36" s="47"/>
+      <c r="D36" s="24" t="s">
+        <v>73</v>
+      </c>
+      <c r="E36" s="28"/>
+      <c r="F36" s="28" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" ht="16.5" thickBot="1">
+      <c r="A37" s="9">
         <v>34</v>
       </c>
-      <c r="B36" s="5" t="s">
-        <v>67</v>
-      </c>
-      <c r="C36" s="6" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="37" spans="1:4" ht="16.5" thickBot="1">
-      <c r="A37" s="9">
+      <c r="B37" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="C37" s="6" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" ht="16.5" thickBot="1">
+      <c r="A38" s="9">
         <v>35</v>
       </c>
-      <c r="B37" s="5" t="s">
-        <v>69</v>
-      </c>
-      <c r="C37" s="6" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="38" spans="1:4" ht="16.5" thickBot="1">
-      <c r="A38" s="9">
+      <c r="B38" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="C38" s="6" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" ht="16.5" thickBot="1">
+      <c r="A39" s="9">
         <v>36</v>
       </c>
-      <c r="B38" s="5" t="s">
-        <v>70</v>
-      </c>
-      <c r="C38" s="6"/>
-      <c r="D38" s="14" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="39" spans="1:4" ht="16.5" thickBot="1">
-      <c r="A39" s="9">
-        <v>37</v>
-      </c>
       <c r="B39" s="5" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="C39" s="6"/>
       <c r="D39" s="14" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="40" spans="1:4" ht="16.5" thickBot="1">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" ht="16.5" thickBot="1">
       <c r="A40" s="9">
+        <v>37</v>
+      </c>
+      <c r="B40" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="C40" s="6"/>
+      <c r="D40" s="14" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" s="28" customFormat="1" ht="16.5" thickBot="1">
+      <c r="A41" s="37">
         <v>38</v>
       </c>
-      <c r="B40" s="5" t="s">
-        <v>74</v>
-      </c>
-      <c r="C40" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="41" spans="1:4" ht="17.100000000000001" customHeight="1" thickBot="1">
-      <c r="A41" s="9">
+      <c r="B41" s="41" t="s">
+        <v>81</v>
+      </c>
+      <c r="C41" s="28" t="s">
+        <v>71</v>
+      </c>
+      <c r="D41" s="28" t="s">
+        <v>82</v>
+      </c>
+      <c r="F41" s="28" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" ht="17.100000000000001" customHeight="1" thickBot="1">
+      <c r="A42" s="9">
         <v>39</v>
       </c>
-      <c r="B41" s="5" t="s">
-        <v>75</v>
-      </c>
-      <c r="C41" s="6" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="42" spans="1:4" ht="16.5" thickBot="1">
-      <c r="A42" s="9">
+      <c r="B42" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="C42" s="6" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" ht="16.5" thickBot="1">
+      <c r="A43" s="9">
         <v>40</v>
       </c>
-      <c r="B42" s="5" t="s">
-        <v>77</v>
-      </c>
-      <c r="C42" s="6" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="43" spans="1:4" ht="16.5" thickBot="1">
-      <c r="A43" s="9">
+      <c r="B43" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="C43" s="6" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" ht="16.5" thickBot="1">
+      <c r="A44" s="9">
         <v>41</v>
       </c>
-      <c r="B43" s="5" t="s">
-        <v>78</v>
-      </c>
-      <c r="C43" s="6" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="44" spans="1:4" ht="16.5" thickBot="1">
-      <c r="A44" s="9">
+      <c r="B44" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="C44" s="6" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" s="28" customFormat="1" ht="15.75">
+      <c r="A45" s="37">
         <v>42</v>
       </c>
-      <c r="B44" s="5" t="s">
-        <v>80</v>
-      </c>
-      <c r="C44" s="6" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="45" spans="1:4" ht="16.5" thickBot="1">
-      <c r="A45" s="9">
+      <c r="B45" s="41" t="s">
+        <v>88</v>
+      </c>
+      <c r="C45" s="42" t="s">
+        <v>71</v>
+      </c>
+      <c r="D45" s="28" t="s">
+        <v>24</v>
+      </c>
+      <c r="F45" s="28" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" ht="16.5" thickBot="1">
+      <c r="A46" s="9">
         <v>43</v>
       </c>
-      <c r="B45" s="5" t="s">
-        <v>81</v>
-      </c>
-      <c r="C45" s="6"/>
-      <c r="D45" s="14" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="46" spans="1:4" ht="15.75">
-      <c r="A46" s="9">
+      <c r="B46" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="C46" s="6"/>
+      <c r="D46" s="14" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" ht="15.75">
+      <c r="A47" s="9">
         <v>44</v>
       </c>
-      <c r="B46" s="5" t="s">
-        <v>82</v>
-      </c>
-      <c r="C46" s="6" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="47" spans="1:4" ht="16.5" thickBot="1">
-      <c r="A47" s="9">
+      <c r="B47" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="C47" s="6" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" ht="16.5" thickBot="1">
+      <c r="A48" s="9">
         <v>45</v>
       </c>
-      <c r="B47" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="C47" s="6" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="48" spans="1:4" ht="16.5" thickBot="1">
-      <c r="A48" s="9">
+      <c r="B48" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="C48" s="6" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" ht="16.5" thickBot="1">
+      <c r="A49" s="9">
         <v>46</v>
       </c>
-      <c r="B48" s="5" t="s">
-        <v>86</v>
-      </c>
-      <c r="C48" s="6" t="s">
-        <v>87</v>
-      </c>
-      <c r="D48" s="14"/>
-    </row>
-    <row r="49" spans="1:4" ht="15.75">
-      <c r="A49" s="9">
+      <c r="B49" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="C49" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="D49" s="14"/>
+    </row>
+    <row r="50" spans="1:6" ht="15.75">
+      <c r="A50" s="9">
         <v>47</v>
       </c>
-      <c r="B49" s="5" t="s">
-        <v>88</v>
-      </c>
-      <c r="C49" s="6"/>
-      <c r="D49" s="14" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="50" spans="1:4" ht="16.5" thickBot="1">
-      <c r="A50" s="9">
-        <v>48</v>
-      </c>
       <c r="B50" s="5" t="s">
-        <v>89</v>
+        <v>96</v>
       </c>
       <c r="C50" s="6"/>
       <c r="D50" s="14" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="51" spans="1:4" ht="15.75">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" ht="16.5" thickBot="1">
       <c r="A51" s="9">
+        <v>48</v>
+      </c>
+      <c r="B51" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="C51" s="6"/>
+      <c r="D51" s="14" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" ht="15.75">
+      <c r="A52" s="9">
         <v>49</v>
       </c>
-      <c r="B51" s="5" t="s">
-        <v>91</v>
-      </c>
-      <c r="C51" s="6" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="52" spans="1:4" ht="15.75">
-      <c r="A52" s="12"/>
-      <c r="B52" t="s">
-        <v>93</v>
-      </c>
-      <c r="C52" s="30" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="53" spans="1:4" ht="15.75">
+      <c r="B52" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C52" s="6" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" ht="15.75">
       <c r="A53" s="12"/>
       <c r="B53" t="s">
-        <v>93</v>
+        <v>25</v>
       </c>
       <c r="C53" s="30" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="54" spans="1:4" ht="15.75">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" ht="15.75">
       <c r="A54" s="12"/>
       <c r="B54" t="s">
-        <v>96</v>
+        <v>25</v>
       </c>
       <c r="C54" s="30" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="55" spans="1:4" ht="15.75">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" ht="15.75">
       <c r="A55" s="12"/>
       <c r="B55" t="s">
-        <v>93</v>
+        <v>103</v>
       </c>
       <c r="C55" s="30" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="56" spans="1:4" ht="15.75">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" ht="15.75">
       <c r="A56" s="12"/>
       <c r="B56" t="s">
-        <v>93</v>
+        <v>25</v>
       </c>
       <c r="C56" s="30" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="57" spans="1:4" ht="15.75">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" ht="15.75">
       <c r="A57" s="12"/>
       <c r="B57" t="s">
-        <v>93</v>
+        <v>25</v>
       </c>
       <c r="C57" s="30" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="58" spans="1:4" ht="15.75">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" ht="15.75">
       <c r="A58" s="12"/>
       <c r="B58" t="s">
-        <v>93</v>
+        <v>25</v>
       </c>
       <c r="C58" s="30" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="59" spans="1:4" ht="15.75">
-      <c r="A59" s="12">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" ht="15.75">
+      <c r="A59" s="12"/>
+      <c r="B59" t="s">
+        <v>25</v>
+      </c>
+      <c r="C59" s="30" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" ht="15.75">
+      <c r="A60" s="12">
         <v>50</v>
       </c>
-      <c r="B59" t="s">
-        <v>102</v>
-      </c>
-      <c r="C59" s="30" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="60" spans="1:4" ht="15.75">
-      <c r="A60" s="12"/>
       <c r="B60" t="s">
-        <v>93</v>
+        <v>109</v>
       </c>
       <c r="C60" s="30" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="61" spans="1:4" ht="15.75">
-      <c r="A61" s="12">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" ht="15.75">
+      <c r="A61" s="12"/>
+      <c r="B61" t="s">
+        <v>25</v>
+      </c>
+      <c r="C61" s="30" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" s="28" customFormat="1" ht="15.75">
+      <c r="A62" s="37">
+        <v>50</v>
+      </c>
+      <c r="B62" s="41" t="s">
+        <v>112</v>
+      </c>
+      <c r="C62" s="28" t="s">
+        <v>111</v>
+      </c>
+      <c r="D62" s="28" t="s">
+        <v>113</v>
+      </c>
+      <c r="F62" s="28" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" s="28" customFormat="1" ht="15.75">
+      <c r="A63" s="44">
         <v>51</v>
       </c>
-      <c r="B61" t="s">
-        <v>105</v>
-      </c>
-      <c r="C61" s="30" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="62" spans="1:4" ht="15.75">
-      <c r="A62" s="12">
-        <f t="shared" ref="A62:A112" si="0">A61+1</f>
+      <c r="B63" s="28" t="s">
+        <v>115</v>
+      </c>
+      <c r="C63" s="28" t="s">
+        <v>116</v>
+      </c>
+      <c r="D63" s="28" t="s">
+        <v>24</v>
+      </c>
+      <c r="F63" s="28" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" ht="15.75">
+      <c r="A64" s="12">
+        <f t="shared" ref="A64:A118" si="0">A63+1</f>
         <v>52</v>
       </c>
-      <c r="B62" s="30" t="s">
-        <v>107</v>
-      </c>
-      <c r="C62" s="30" t="s">
-        <v>108</v>
-      </c>
-      <c r="D62" s="30"/>
-    </row>
-    <row r="63" spans="1:4" ht="15.75">
-      <c r="A63" s="12">
-        <f t="shared" si="0"/>
-        <v>53</v>
-      </c>
-      <c r="B63" s="30" t="s">
-        <v>109</v>
-      </c>
-      <c r="C63" s="30" t="s">
-        <v>110</v>
-      </c>
-      <c r="D63" s="30"/>
-    </row>
-    <row r="64" spans="1:4" ht="15.75">
-      <c r="A64" s="12">
-        <f t="shared" si="0"/>
-        <v>54</v>
-      </c>
       <c r="B64" s="30" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="C64" s="30" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="D64" s="30"/>
     </row>
     <row r="65" spans="1:6" ht="15.75">
       <c r="A65" s="12">
         <f t="shared" si="0"/>
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B65" s="30" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="C65" s="30" t="s">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="D65" s="30"/>
     </row>
     <row r="66" spans="1:6" ht="15.75">
       <c r="A66" s="12">
         <f t="shared" si="0"/>
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B66" s="30" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="C66" s="30" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="D66" s="30"/>
     </row>
     <row r="67" spans="1:6" ht="15.75">
       <c r="A67" s="12">
         <f t="shared" si="0"/>
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B67" s="30" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="C67" s="30" t="s">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="D67" s="30"/>
     </row>
     <row r="68" spans="1:6" ht="15.75">
       <c r="A68" s="12">
         <f t="shared" si="0"/>
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B68" s="30" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="C68" s="30" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="D68" s="30"/>
     </row>
     <row r="69" spans="1:6" ht="15.75">
       <c r="A69" s="12">
+        <f>A68+1</f>
+        <v>57</v>
+      </c>
+      <c r="B69" s="30" t="s">
+        <v>127</v>
+      </c>
+      <c r="C69" s="30" t="s">
+        <v>128</v>
+      </c>
+      <c r="D69" s="30"/>
+    </row>
+    <row r="70" spans="1:6" s="28" customFormat="1" ht="15.75">
+      <c r="A70" s="44">
         <f t="shared" si="0"/>
-        <v>59</v>
-      </c>
-      <c r="B69" s="30" t="s">
-        <v>121</v>
-      </c>
-      <c r="C69" s="30" t="s">
-        <v>122</v>
-      </c>
-      <c r="D69" s="30"/>
-    </row>
-    <row r="70" spans="1:6" ht="15.75">
-      <c r="A70" s="12">
-        <f t="shared" si="0"/>
-        <v>60</v>
-      </c>
-      <c r="B70" s="30" t="s">
-        <v>123</v>
-      </c>
-      <c r="C70" s="30" t="s">
-        <v>124</v>
-      </c>
-      <c r="D70" s="30"/>
+        <v>58</v>
+      </c>
+      <c r="B70" s="28" t="s">
+        <v>129</v>
+      </c>
+      <c r="C70" s="28" t="s">
+        <v>130</v>
+      </c>
+      <c r="D70" s="28" t="s">
+        <v>131</v>
+      </c>
+      <c r="F70" s="28" t="s">
+        <v>25</v>
+      </c>
     </row>
     <row r="71" spans="1:6" ht="15.75">
       <c r="A71" s="12">
         <f t="shared" si="0"/>
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B71" s="30" t="s">
-        <v>125</v>
+        <v>132</v>
       </c>
       <c r="C71" s="30" t="s">
-        <v>126</v>
+        <v>133</v>
       </c>
       <c r="D71" s="30"/>
     </row>
     <row r="72" spans="1:6" ht="15.75">
       <c r="A72" s="12">
         <f t="shared" si="0"/>
-        <v>62</v>
-      </c>
-      <c r="B72" s="29" t="s">
-        <v>127</v>
+        <v>60</v>
+      </c>
+      <c r="B72" s="30" t="s">
+        <v>134</v>
       </c>
       <c r="C72" s="30" t="s">
-        <v>128</v>
-      </c>
-      <c r="D72" s="29"/>
-      <c r="F72" t="s">
-        <v>129</v>
-      </c>
+        <v>135</v>
+      </c>
+      <c r="D72" s="30"/>
     </row>
     <row r="73" spans="1:6" ht="15.75">
       <c r="A73" s="12">
         <f t="shared" si="0"/>
+        <v>61</v>
+      </c>
+      <c r="B73" s="30" t="s">
+        <v>136</v>
+      </c>
+      <c r="C73" s="30" t="s">
+        <v>137</v>
+      </c>
+      <c r="D73" s="30"/>
+    </row>
+    <row r="74" spans="1:6" ht="15.75">
+      <c r="A74" s="12">
+        <f t="shared" si="0"/>
+        <v>62</v>
+      </c>
+      <c r="B74" s="29" t="s">
+        <v>20</v>
+      </c>
+      <c r="C74" s="30" t="s">
+        <v>138</v>
+      </c>
+      <c r="D74" s="29"/>
+      <c r="F74" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" ht="15.75">
+      <c r="A75" s="12">
+        <f t="shared" si="0"/>
         <v>63</v>
       </c>
-      <c r="B73" s="5" t="s">
-        <v>130</v>
-      </c>
-      <c r="C73" s="30" t="s">
-        <v>131</v>
-      </c>
-      <c r="D73" s="5"/>
-    </row>
-    <row r="74" spans="1:6" ht="15.75">
-      <c r="A74" s="12"/>
-      <c r="B74" t="s">
-        <v>93</v>
-      </c>
-      <c r="C74" s="30" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="75" spans="1:6" ht="15.75">
-      <c r="A75" s="12"/>
       <c r="B75" t="s">
-        <v>93</v>
+        <v>140</v>
       </c>
       <c r="C75" s="30" t="s">
-        <v>133</v>
-      </c>
+        <v>141</v>
+      </c>
+      <c r="D75" s="5"/>
     </row>
     <row r="76" spans="1:6" ht="15.75">
       <c r="A76" s="12"/>
       <c r="B76" t="s">
-        <v>93</v>
+        <v>25</v>
       </c>
       <c r="C76" s="30" t="s">
-        <v>134</v>
+        <v>142</v>
       </c>
     </row>
     <row r="77" spans="1:6" ht="15.75">
       <c r="A77" s="12"/>
       <c r="B77" t="s">
-        <v>93</v>
+        <v>25</v>
       </c>
       <c r="C77" s="30" t="s">
-        <v>135</v>
+        <v>143</v>
       </c>
     </row>
     <row r="78" spans="1:6" ht="15.75">
       <c r="A78" s="12"/>
       <c r="B78" t="s">
-        <v>93</v>
+        <v>25</v>
       </c>
       <c r="C78" s="30" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
     </row>
     <row r="79" spans="1:6" ht="15.75">
       <c r="A79" s="12"/>
       <c r="B79" t="s">
-        <v>93</v>
+        <v>25</v>
       </c>
       <c r="C79" s="30" t="s">
-        <v>137</v>
+        <v>145</v>
       </c>
     </row>
     <row r="80" spans="1:6" ht="15.75">
       <c r="A80" s="12"/>
       <c r="B80" t="s">
-        <v>138</v>
+        <v>25</v>
       </c>
       <c r="C80" s="30" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="81" spans="1:4" ht="15.75">
-      <c r="A81" s="12">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" ht="15.75">
+      <c r="A81" s="12"/>
+      <c r="B81" t="s">
+        <v>25</v>
+      </c>
+      <c r="C81" s="30" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" ht="15.75">
+      <c r="A82" s="12"/>
+      <c r="B82" t="s">
+        <v>148</v>
+      </c>
+      <c r="C82" s="30" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" ht="15.75">
+      <c r="A83" s="12">
         <v>64</v>
       </c>
-      <c r="B81" t="s">
-        <v>140</v>
-      </c>
-      <c r="C81" s="30" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="82" spans="1:4" ht="15.75">
-      <c r="A82" s="12">
-        <f t="shared" si="0"/>
+      <c r="B83" t="s">
+        <v>150</v>
+      </c>
+      <c r="C83" s="30" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" s="28" customFormat="1" ht="15.75">
+      <c r="A84" s="37">
+        <v>64</v>
+      </c>
+      <c r="B84" s="28" t="s">
+        <v>152</v>
+      </c>
+      <c r="C84" s="28" t="s">
+        <v>151</v>
+      </c>
+      <c r="D84" s="28" t="s">
+        <v>153</v>
+      </c>
+      <c r="F84" s="28" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" ht="15.75">
+      <c r="A85" s="12">
+        <f>A83+1</f>
         <v>65</v>
       </c>
-      <c r="B82" t="s">
-        <v>142</v>
-      </c>
-      <c r="C82" s="30" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="83" spans="1:4" ht="15.75">
-      <c r="A83" s="12">
-        <f t="shared" si="0"/>
+      <c r="B85" t="s">
+        <v>154</v>
+      </c>
+      <c r="C85" s="30" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" s="28" customFormat="1" ht="15.75">
+      <c r="A86" s="37">
+        <v>65</v>
+      </c>
+      <c r="B86" s="41" t="s">
+        <v>156</v>
+      </c>
+      <c r="C86" s="28" t="s">
+        <v>155</v>
+      </c>
+      <c r="D86" s="28" t="s">
+        <v>157</v>
+      </c>
+      <c r="F86" s="28" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" ht="15.75">
+      <c r="A87" s="12">
+        <f>A85+1</f>
         <v>66</v>
       </c>
-      <c r="B83" s="30" t="s">
-        <v>144</v>
-      </c>
-      <c r="C83" s="30" t="s">
-        <v>145</v>
-      </c>
-      <c r="D83" s="30"/>
-    </row>
-    <row r="84" spans="1:4" ht="15.75">
-      <c r="A84" s="12">
+      <c r="B87" s="30" t="s">
+        <v>158</v>
+      </c>
+      <c r="C87" s="30" t="s">
+        <v>159</v>
+      </c>
+      <c r="D87" s="30"/>
+    </row>
+    <row r="88" spans="1:6" ht="15.75">
+      <c r="A88" s="12">
         <f t="shared" si="0"/>
         <v>67</v>
       </c>
-      <c r="B84" s="30" t="s">
-        <v>146</v>
-      </c>
-      <c r="C84" s="30" t="s">
-        <v>147</v>
-      </c>
-      <c r="D84" s="30"/>
-    </row>
-    <row r="85" spans="1:4" ht="15.75">
-      <c r="A85" s="12">
+      <c r="B88" s="30" t="s">
+        <v>160</v>
+      </c>
+      <c r="C88" s="30" t="s">
+        <v>161</v>
+      </c>
+      <c r="D88" s="30"/>
+    </row>
+    <row r="89" spans="1:6" ht="15.75">
+      <c r="A89" s="12">
         <f t="shared" si="0"/>
         <v>68</v>
       </c>
-      <c r="B85" s="30" t="s">
-        <v>148</v>
-      </c>
-      <c r="C85" s="30" t="s">
-        <v>149</v>
-      </c>
-      <c r="D85" s="30"/>
-    </row>
-    <row r="86" spans="1:4" ht="15.75">
-      <c r="A86" s="12">
+      <c r="B89" s="30" t="s">
+        <v>162</v>
+      </c>
+      <c r="C89" s="30" t="s">
+        <v>163</v>
+      </c>
+      <c r="D89" s="30"/>
+    </row>
+    <row r="90" spans="1:6" ht="15.75">
+      <c r="A90" s="12">
         <f t="shared" si="0"/>
         <v>69</v>
       </c>
-      <c r="B86" s="30" t="s">
-        <v>150</v>
-      </c>
-      <c r="C86" s="30" t="s">
-        <v>151</v>
-      </c>
-      <c r="D86" s="30"/>
-    </row>
-    <row r="87" spans="1:4" ht="15.75">
-      <c r="A87" s="12">
+      <c r="B90" s="30" t="s">
+        <v>164</v>
+      </c>
+      <c r="C90" s="30" t="s">
+        <v>165</v>
+      </c>
+      <c r="D90" s="30"/>
+    </row>
+    <row r="91" spans="1:6" ht="15.75">
+      <c r="A91" s="12">
         <f t="shared" si="0"/>
         <v>70</v>
       </c>
-      <c r="B87" s="30" t="s">
-        <v>152</v>
-      </c>
-      <c r="C87" s="30" t="s">
-        <v>153</v>
-      </c>
-      <c r="D87" s="30"/>
-    </row>
-    <row r="88" spans="1:4" ht="15.75">
-      <c r="A88" s="12">
+      <c r="B91" s="30" t="s">
+        <v>166</v>
+      </c>
+      <c r="C91" s="30" t="s">
+        <v>167</v>
+      </c>
+      <c r="D91" s="30"/>
+    </row>
+    <row r="92" spans="1:6" ht="15.75">
+      <c r="A92" s="12">
         <f t="shared" si="0"/>
         <v>71</v>
       </c>
-      <c r="B88" s="30" t="s">
-        <v>102</v>
-      </c>
-      <c r="C88" s="30" t="s">
-        <v>154</v>
-      </c>
-      <c r="D88" s="30"/>
-    </row>
-    <row r="89" spans="1:4" ht="15.75">
-      <c r="A89" s="12">
+      <c r="B92" s="30" t="s">
+        <v>109</v>
+      </c>
+      <c r="C92" s="30" t="s">
+        <v>168</v>
+      </c>
+      <c r="D92" s="30"/>
+    </row>
+    <row r="93" spans="1:6" ht="15.75">
+      <c r="A93" s="12">
         <f t="shared" si="0"/>
         <v>72</v>
       </c>
-      <c r="B89" t="s">
-        <v>155</v>
-      </c>
-      <c r="C89" s="30" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="90" spans="1:4" ht="15.75">
-      <c r="A90" s="12">
-        <f t="shared" si="0"/>
+      <c r="B93" t="s">
+        <v>169</v>
+      </c>
+      <c r="C93" s="30" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6" s="28" customFormat="1" ht="15.75">
+      <c r="A94" s="37">
+        <v>72</v>
+      </c>
+      <c r="B94" s="41" t="s">
+        <v>171</v>
+      </c>
+      <c r="C94" s="28" t="s">
+        <v>170</v>
+      </c>
+      <c r="D94" s="28" t="s">
+        <v>172</v>
+      </c>
+      <c r="F94" s="28" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6" ht="15.75">
+      <c r="A95" s="12">
+        <f>A93+1</f>
         <v>73</v>
       </c>
-      <c r="B90" s="30" t="s">
-        <v>157</v>
-      </c>
-      <c r="C90" s="30" t="s">
-        <v>158</v>
-      </c>
-      <c r="D90" s="30"/>
-    </row>
-    <row r="91" spans="1:4" ht="15.75">
-      <c r="A91" s="12">
+      <c r="B95" s="30" t="s">
+        <v>173</v>
+      </c>
+      <c r="C95" s="30" t="s">
+        <v>174</v>
+      </c>
+      <c r="D95" s="30"/>
+    </row>
+    <row r="96" spans="1:6" ht="15.75">
+      <c r="A96" s="12">
         <f t="shared" si="0"/>
         <v>74</v>
       </c>
-      <c r="B91" s="30" t="s">
-        <v>159</v>
-      </c>
-      <c r="C91" s="30" t="s">
-        <v>160</v>
-      </c>
-      <c r="D91" s="30"/>
-    </row>
-    <row r="92" spans="1:4" ht="15.75">
-      <c r="A92" s="12">
+      <c r="B96" s="30" t="s">
+        <v>175</v>
+      </c>
+      <c r="C96" s="30" t="s">
+        <v>176</v>
+      </c>
+      <c r="D96" s="30"/>
+    </row>
+    <row r="97" spans="1:6" ht="15.75">
+      <c r="A97" s="12">
         <f t="shared" si="0"/>
         <v>75</v>
       </c>
-      <c r="B92" s="30" t="s">
-        <v>161</v>
-      </c>
-      <c r="C92" s="30" t="s">
-        <v>162</v>
-      </c>
-      <c r="D92" s="30"/>
-    </row>
-    <row r="93" spans="1:4" ht="15.75">
-      <c r="A93" s="12">
+      <c r="B97" s="30" t="s">
+        <v>177</v>
+      </c>
+      <c r="C97" s="30" t="s">
+        <v>178</v>
+      </c>
+      <c r="D97" s="30"/>
+    </row>
+    <row r="98" spans="1:6" ht="15.75">
+      <c r="A98" s="12">
         <v>76</v>
       </c>
-      <c r="B93" s="30" t="s">
-        <v>163</v>
-      </c>
-      <c r="C93" s="30" t="s">
-        <v>164</v>
-      </c>
-      <c r="D93" s="30"/>
-    </row>
-    <row r="94" spans="1:4" ht="15.75">
-      <c r="A94" s="12">
+      <c r="B98" s="30" t="s">
+        <v>179</v>
+      </c>
+      <c r="C98" s="30" t="s">
+        <v>180</v>
+      </c>
+      <c r="D98" s="30"/>
+    </row>
+    <row r="99" spans="1:6" ht="15.75">
+      <c r="A99" s="12">
         <f t="shared" si="0"/>
         <v>77</v>
       </c>
-      <c r="B94" s="30" t="s">
-        <v>165</v>
-      </c>
-      <c r="C94" s="30" t="s">
-        <v>166</v>
-      </c>
-      <c r="D94" s="30"/>
-    </row>
-    <row r="95" spans="1:4" ht="15.75">
-      <c r="A95" s="12">
+      <c r="B99" s="30" t="s">
+        <v>181</v>
+      </c>
+      <c r="C99" s="30" t="s">
+        <v>182</v>
+      </c>
+      <c r="D99" s="30"/>
+    </row>
+    <row r="100" spans="1:6" ht="15.75">
+      <c r="A100" s="12">
         <f t="shared" si="0"/>
         <v>78</v>
       </c>
-      <c r="B95" t="s">
-        <v>167</v>
-      </c>
-      <c r="C95" s="30" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="96" spans="1:4" ht="15.75">
-      <c r="A96" s="12">
-        <f t="shared" si="0"/>
+      <c r="B100" t="s">
+        <v>183</v>
+      </c>
+      <c r="C100" s="30" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="101" spans="1:6" s="28" customFormat="1" ht="15.75">
+      <c r="A101" s="37">
+        <v>78</v>
+      </c>
+      <c r="B101" s="41" t="s">
+        <v>185</v>
+      </c>
+      <c r="C101" s="28" t="s">
+        <v>184</v>
+      </c>
+      <c r="D101" s="28" t="s">
+        <v>186</v>
+      </c>
+      <c r="F101" s="28" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="102" spans="1:6" ht="15.75">
+      <c r="A102" s="12">
+        <f>A100+1</f>
         <v>79</v>
       </c>
-      <c r="B96" s="30" t="s">
-        <v>169</v>
-      </c>
-      <c r="C96" s="30" t="s">
-        <v>170</v>
-      </c>
-      <c r="D96" s="30"/>
-    </row>
-    <row r="97" spans="1:4" ht="15.75">
-      <c r="A97" s="12">
+      <c r="B102" s="30" t="s">
+        <v>187</v>
+      </c>
+      <c r="C102" s="30" t="s">
+        <v>188</v>
+      </c>
+      <c r="D102" s="30"/>
+    </row>
+    <row r="103" spans="1:6" ht="15.75">
+      <c r="A103" s="12">
         <f t="shared" si="0"/>
         <v>80</v>
       </c>
-      <c r="B97" s="30" t="s">
-        <v>171</v>
-      </c>
-      <c r="C97" s="30" t="s">
-        <v>172</v>
-      </c>
-      <c r="D97" s="30"/>
-    </row>
-    <row r="98" spans="1:4" ht="15.75">
-      <c r="A98" s="12">
+      <c r="B103" s="30" t="s">
+        <v>189</v>
+      </c>
+      <c r="C103" s="30" t="s">
+        <v>190</v>
+      </c>
+      <c r="D103" s="30"/>
+    </row>
+    <row r="104" spans="1:6" ht="15.75">
+      <c r="A104" s="12">
         <f t="shared" si="0"/>
         <v>81</v>
       </c>
-      <c r="B98" s="30" t="s">
-        <v>173</v>
-      </c>
-      <c r="C98" s="30" t="s">
-        <v>174</v>
-      </c>
-      <c r="D98" s="30"/>
-    </row>
-    <row r="99" spans="1:4" ht="15.75">
-      <c r="A99" s="12">
+      <c r="B104" s="30" t="s">
+        <v>191</v>
+      </c>
+      <c r="C104" s="30" t="s">
+        <v>192</v>
+      </c>
+      <c r="D104" s="30"/>
+    </row>
+    <row r="105" spans="1:6" ht="15.75">
+      <c r="A105" s="12">
         <f t="shared" si="0"/>
         <v>82</v>
       </c>
-      <c r="B99" s="30" t="s">
-        <v>175</v>
-      </c>
-      <c r="C99" s="30" t="s">
-        <v>176</v>
-      </c>
-      <c r="D99" s="30"/>
-    </row>
-    <row r="100" spans="1:4" ht="15.75">
-      <c r="A100" s="12">
+      <c r="B105" s="30" t="s">
+        <v>193</v>
+      </c>
+      <c r="C105" s="30" t="s">
+        <v>194</v>
+      </c>
+      <c r="D105" s="30"/>
+    </row>
+    <row r="106" spans="1:6" ht="15.75">
+      <c r="A106" s="12">
         <f t="shared" si="0"/>
         <v>83</v>
       </c>
-      <c r="B100" s="30" t="s">
-        <v>177</v>
-      </c>
-      <c r="C100" s="30" t="s">
-        <v>178</v>
-      </c>
-      <c r="D100" s="30"/>
-    </row>
-    <row r="101" spans="1:4" ht="15.75">
-      <c r="A101" s="12">
+      <c r="B106" s="30" t="s">
+        <v>195</v>
+      </c>
+      <c r="C106" s="30" t="s">
+        <v>196</v>
+      </c>
+      <c r="D106" s="30"/>
+    </row>
+    <row r="107" spans="1:6" ht="15.75">
+      <c r="A107" s="12">
         <f t="shared" si="0"/>
         <v>84</v>
       </c>
-      <c r="B101" t="s">
-        <v>179</v>
-      </c>
-      <c r="C101" s="30" t="s">
-        <v>180</v>
-      </c>
-      <c r="D101" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="102" spans="1:4" ht="15.75">
-      <c r="A102" s="12">
+      <c r="B107" t="s">
+        <v>197</v>
+      </c>
+      <c r="C107" s="30" t="s">
+        <v>198</v>
+      </c>
+      <c r="D107" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="108" spans="1:6" ht="15.75">
+      <c r="A108" s="12">
         <f t="shared" si="0"/>
         <v>85</v>
       </c>
-      <c r="B102" t="s">
-        <v>182</v>
-      </c>
-      <c r="C102" s="30" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="103" spans="1:4" ht="15.75">
-      <c r="A103" s="12">
+      <c r="B108" t="s">
+        <v>200</v>
+      </c>
+      <c r="C108" s="30" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="109" spans="1:6" ht="15.75">
+      <c r="A109" s="12">
         <f t="shared" si="0"/>
         <v>86</v>
       </c>
-      <c r="B103" t="s">
-        <v>184</v>
-      </c>
-      <c r="C103" s="30" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="104" spans="1:4" ht="15.75">
-      <c r="A104" s="12"/>
-      <c r="B104" t="s">
-        <v>93</v>
-      </c>
-      <c r="C104" s="30" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="105" spans="1:4" ht="15.75">
-      <c r="A105" s="12"/>
-      <c r="B105" t="s">
-        <v>93</v>
-      </c>
-      <c r="C105" s="30" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="106" spans="1:4" ht="15.75">
-      <c r="A106" s="12">
+      <c r="B109" t="s">
+        <v>202</v>
+      </c>
+      <c r="C109" s="30" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="110" spans="1:6" ht="15.75">
+      <c r="A110" s="12"/>
+      <c r="B110" t="s">
+        <v>25</v>
+      </c>
+      <c r="C110" s="30" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="111" spans="1:6" ht="15.75">
+      <c r="A111" s="12"/>
+      <c r="B111" t="s">
+        <v>25</v>
+      </c>
+      <c r="C111" s="30" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="112" spans="1:6" ht="15.75">
+      <c r="A112" s="12">
         <v>87</v>
       </c>
-      <c r="B106" t="s">
-        <v>188</v>
-      </c>
-      <c r="C106" s="30" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="107" spans="1:4" ht="15.75">
-      <c r="A107" s="12">
+      <c r="B112" t="s">
+        <v>206</v>
+      </c>
+      <c r="C112" s="30" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="113" spans="1:6" ht="15.75">
+      <c r="A113" s="12">
         <f t="shared" si="0"/>
         <v>88</v>
       </c>
-      <c r="B107" t="s">
-        <v>190</v>
-      </c>
-      <c r="C107" s="30" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="108" spans="1:4" ht="15.75">
-      <c r="A108" s="9">
+      <c r="B113" t="s">
+        <v>208</v>
+      </c>
+      <c r="C113" s="30" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="114" spans="1:6" s="28" customFormat="1" ht="15.75">
+      <c r="A114" s="37">
         <v>89</v>
       </c>
-      <c r="B108" s="29" t="s">
-        <v>192</v>
-      </c>
-      <c r="C108" s="30" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="109" spans="1:4" ht="15.75">
-      <c r="A109" s="12">
+      <c r="B114" s="45" t="s">
+        <v>210</v>
+      </c>
+      <c r="C114" s="28" t="s">
+        <v>209</v>
+      </c>
+      <c r="D114" s="28" t="s">
+        <v>24</v>
+      </c>
+      <c r="F114" s="28" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="115" spans="1:6" s="28" customFormat="1" ht="15.75">
+      <c r="A115" s="44">
         <f t="shared" si="0"/>
         <v>90</v>
       </c>
-      <c r="B109" s="29" t="s">
-        <v>193</v>
-      </c>
-      <c r="C109" s="30" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="110" spans="1:4" ht="15.75">
-      <c r="A110" s="12"/>
-      <c r="B110" s="29" t="s">
-        <v>93</v>
-      </c>
-      <c r="C110" s="30" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="111" spans="1:4" ht="15.75">
-      <c r="A111" s="12">
+      <c r="B115" s="45" t="s">
+        <v>211</v>
+      </c>
+      <c r="C115" s="28" t="s">
+        <v>212</v>
+      </c>
+      <c r="D115" s="28" t="s">
+        <v>24</v>
+      </c>
+      <c r="F115" s="28" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="116" spans="1:6" ht="15.75">
+      <c r="A116" s="12"/>
+      <c r="B116" s="29" t="s">
+        <v>25</v>
+      </c>
+      <c r="C116" s="30" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="117" spans="1:6" ht="15.75">
+      <c r="A117" s="12">
         <v>91</v>
       </c>
-      <c r="B111" s="29" t="s">
-        <v>196</v>
-      </c>
-      <c r="C111" s="30" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="112" spans="1:4" ht="15.75">
-      <c r="A112" s="12">
+      <c r="B117" s="29" t="s">
+        <v>214</v>
+      </c>
+      <c r="C117" s="30" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="118" spans="1:6" s="28" customFormat="1" ht="15.75">
+      <c r="A118" s="44">
         <f t="shared" si="0"/>
         <v>92</v>
       </c>
-      <c r="B112" t="s">
-        <v>198</v>
-      </c>
-      <c r="C112" s="30" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="113" spans="1:3" ht="15.75">
-      <c r="A113" s="9">
+      <c r="B118" s="28" t="s">
+        <v>81</v>
+      </c>
+      <c r="C118" s="28" t="s">
+        <v>69</v>
+      </c>
+      <c r="D118" s="28" t="s">
+        <v>24</v>
+      </c>
+      <c r="F118" s="28" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="119" spans="1:6" ht="15.75">
+      <c r="A119" s="9">
         <v>93</v>
       </c>
-      <c r="B113" s="31" t="s">
-        <v>199</v>
-      </c>
-      <c r="C113" s="30" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="114" spans="1:3" ht="15.75">
-      <c r="A114" s="9"/>
-      <c r="B114" t="s">
-        <v>93</v>
-      </c>
-      <c r="C114" s="30" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="115" spans="1:3" ht="15.75">
-      <c r="A115" s="1"/>
-    </row>
-    <row r="116" spans="1:3" ht="16.5" thickBot="1">
-      <c r="A116" s="1"/>
-    </row>
-    <row r="117" spans="1:3" ht="16.5" thickBot="1">
-      <c r="A117" s="1"/>
-    </row>
-    <row r="118" spans="1:3" ht="16.5" thickBot="1">
-      <c r="A118" s="1"/>
-    </row>
-    <row r="119" spans="1:3" ht="16.5" thickBot="1">
-      <c r="A119" s="1"/>
-    </row>
-    <row r="120" spans="1:3" ht="16.5" thickBot="1">
-      <c r="A120" s="1"/>
-    </row>
-    <row r="121" spans="1:3" ht="16.5" thickBot="1">
+      <c r="B119" s="31" t="s">
+        <v>68</v>
+      </c>
+      <c r="C119" s="30" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="120" spans="1:6" ht="15.75">
+      <c r="A120" s="9"/>
+      <c r="B120" t="s">
+        <v>25</v>
+      </c>
+      <c r="C120" s="30" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="121" spans="1:6" ht="15.75">
       <c r="A121" s="1"/>
     </row>
-    <row r="122" spans="1:3" ht="16.5" thickBot="1">
+    <row r="122" spans="1:6" ht="16.5" thickBot="1">
       <c r="A122" s="1"/>
     </row>
-    <row r="123" spans="1:3" ht="16.5" thickBot="1">
+    <row r="123" spans="1:6" ht="16.5" thickBot="1">
       <c r="A123" s="1"/>
     </row>
-    <row r="124" spans="1:3" ht="16.5" thickBot="1">
+    <row r="124" spans="1:6" ht="16.5" thickBot="1">
       <c r="A124" s="1"/>
     </row>
-    <row r="125" spans="1:3" ht="16.5" thickBot="1">
+    <row r="125" spans="1:6" ht="16.5" thickBot="1">
       <c r="A125" s="1"/>
     </row>
-    <row r="126" spans="1:3" ht="16.5" thickBot="1">
+    <row r="126" spans="1:6" ht="16.5" thickBot="1">
       <c r="A126" s="1"/>
     </row>
-    <row r="127" spans="1:3" ht="15.75"/>
-    <row r="128" spans="1:3" ht="15.75"/>
-    <row r="129" ht="15.75"/>
-    <row r="130" ht="15.75"/>
-    <row r="131" ht="15.75"/>
-    <row r="132" ht="15.75"/>
-    <row r="133" ht="15.75"/>
-    <row r="134" ht="15.75"/>
-    <row r="135" ht="15.75"/>
-    <row r="136" ht="15.75"/>
-    <row r="137" ht="15.75"/>
-    <row r="138" ht="15.75"/>
-    <row r="139" ht="15.75"/>
-    <row r="140" ht="15.75"/>
-    <row r="142" ht="15.75"/>
+    <row r="127" spans="1:6" ht="16.5" thickBot="1">
+      <c r="A127" s="1"/>
+    </row>
+    <row r="128" spans="1:6" ht="16.5" thickBot="1">
+      <c r="A128" s="1"/>
+    </row>
+    <row r="129" spans="1:1" ht="16.5" thickBot="1">
+      <c r="A129" s="1"/>
+    </row>
+    <row r="130" spans="1:1" ht="16.5" thickBot="1">
+      <c r="A130" s="1"/>
+    </row>
+    <row r="131" spans="1:1" ht="16.5" thickBot="1">
+      <c r="A131" s="1"/>
+    </row>
+    <row r="132" spans="1:1" ht="16.5" thickBot="1">
+      <c r="A132" s="1"/>
+    </row>
+    <row r="133" spans="1:1" ht="15.75"/>
+    <row r="134" spans="1:1" ht="15.75"/>
+    <row r="135" spans="1:1" ht="15.75"/>
+    <row r="136" spans="1:1" ht="15.75"/>
+    <row r="137" spans="1:1" ht="15.75"/>
+    <row r="138" spans="1:1" ht="15.75"/>
+    <row r="139" spans="1:1" ht="15.75"/>
+    <row r="140" spans="1:1" ht="15.75"/>
+    <row r="141" spans="1:1" ht="15.75"/>
+    <row r="142" spans="1:1" ht="15.75"/>
+    <row r="143" spans="1:1" ht="15.75"/>
+    <row r="144" spans="1:1" ht="15.75"/>
+    <row r="145" ht="15.75"/>
+    <row r="146" ht="15.75"/>
+    <row r="148" ht="15.75"/>
   </sheetData>
   <phoneticPr fontId="8" type="noConversion"/>
-  <conditionalFormatting sqref="E2:E52 E55:E58 E60:E78 E80:E81 E83:E114">
-    <cfRule type="expression" dxfId="24" priority="1">
+  <conditionalFormatting sqref="E2:E53 E56:E59 E82:E84 E87:E120 E61:E74 E76:E80">
+    <cfRule type="expression" dxfId="25" priority="1">
       <formula>AND($B2&lt;&gt;"",OR($C2&lt;&gt;"",$D2&lt;&gt;""))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E53">
-    <cfRule type="expression" dxfId="23" priority="5">
-      <formula>AND($B53&lt;&gt;"",OR($C53&lt;&gt;"",$D54&lt;&gt;""))</formula>
+  <conditionalFormatting sqref="E54">
+    <cfRule type="expression" dxfId="24" priority="5">
+      <formula>AND($B54&lt;&gt;"",OR($C54&lt;&gt;"",$D55&lt;&gt;""))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E54">
-    <cfRule type="expression" dxfId="22" priority="6">
-      <formula>AND($B54&lt;&gt;"",OR($C54&lt;&gt;"",#REF!&lt;&gt;""))</formula>
+  <conditionalFormatting sqref="E55">
+    <cfRule type="expression" dxfId="23" priority="6">
+      <formula>AND($B55&lt;&gt;"",OR($C55&lt;&gt;"",#REF!&lt;&gt;""))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E59">
-    <cfRule type="expression" dxfId="21" priority="8">
-      <formula>AND($D59&lt;&gt;"",OR($C59&lt;&gt;"",#REF!&lt;&gt;""))</formula>
+  <conditionalFormatting sqref="E60">
+    <cfRule type="expression" dxfId="22" priority="8">
+      <formula>AND($D60&lt;&gt;"",OR($C60&lt;&gt;"",#REF!&lt;&gt;""))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E82">
-    <cfRule type="expression" dxfId="20" priority="10">
-      <formula>AND($B82&lt;&gt;"",OR($C82&lt;&gt;"",$D79&lt;&gt;""))</formula>
+  <conditionalFormatting sqref="E85:E86">
+    <cfRule type="expression" dxfId="21" priority="10">
+      <formula>AND($B85&lt;&gt;"",OR($C85&lt;&gt;"",$D81&lt;&gt;""))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E79">
-    <cfRule type="expression" dxfId="19" priority="11">
-      <formula>AND($B79&lt;&gt;"",OR($C79&lt;&gt;"",#REF!&lt;&gt;""))</formula>
+  <conditionalFormatting sqref="E81">
+    <cfRule type="expression" dxfId="20" priority="11">
+      <formula>AND($B81&lt;&gt;"",OR($C81&lt;&gt;"",#REF!&lt;&gt;""))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E75">
+    <cfRule type="expression" dxfId="19" priority="13">
+      <formula>AND(#REF!&lt;&gt;"",OR($C75&lt;&gt;"",$D75&lt;&gt;""))</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D73 B73" xr:uid="{7139A785-83F1-4465-8349-9788272C85AB}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D75" xr:uid="{7139A785-83F1-4465-8349-9788272C85AB}">
       <formula1>#REF!</formula1>
     </dataValidation>
   </dataValidations>
@@ -3288,10 +3573,10 @@
         <v>3</v>
       </c>
       <c r="E1" s="19" t="s">
-        <v>201</v>
+        <v>217</v>
       </c>
       <c r="F1" s="24" t="s">
-        <v>202</v>
+        <v>218</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="15.75">
@@ -3300,10 +3585,10 @@
       </c>
       <c r="B2" s="12"/>
       <c r="C2" s="2" t="s">
-        <v>203</v>
+        <v>219</v>
       </c>
       <c r="D2" s="13" t="s">
-        <v>204</v>
+        <v>220</v>
       </c>
       <c r="F2" s="24"/>
     </row>
@@ -3313,7 +3598,7 @@
       </c>
       <c r="B3" s="4"/>
       <c r="C3" s="3" t="s">
-        <v>205</v>
+        <v>221</v>
       </c>
       <c r="D3" s="14"/>
     </row>
@@ -3322,13 +3607,13 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>206</v>
+        <v>222</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D4" t="s">
-        <v>207</v>
+        <v>223</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -3336,13 +3621,13 @@
         <v>3</v>
       </c>
       <c r="B5" s="25" t="s">
-        <v>208</v>
+        <v>224</v>
       </c>
       <c r="C5" s="18" t="s">
-        <v>209</v>
+        <v>225</v>
       </c>
       <c r="D5" t="s">
-        <v>210</v>
+        <v>226</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -3350,13 +3635,13 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>211</v>
+        <v>227</v>
       </c>
       <c r="C6" s="18" t="s">
-        <v>212</v>
+        <v>228</v>
       </c>
       <c r="D6" t="s">
-        <v>213</v>
+        <v>229</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="15.95">
@@ -3364,13 +3649,13 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>214</v>
+        <v>230</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>215</v>
+        <v>231</v>
       </c>
       <c r="D7" t="s">
-        <v>216</v>
+        <v>232</v>
       </c>
     </row>
   </sheetData>
@@ -3411,10 +3696,10 @@
         <v>3</v>
       </c>
       <c r="E1" s="23" t="s">
-        <v>201</v>
+        <v>217</v>
       </c>
       <c r="F1" s="24" t="s">
-        <v>202</v>
+        <v>218</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="15.75">
@@ -3423,10 +3708,10 @@
       </c>
       <c r="B2" s="12"/>
       <c r="C2" s="2" t="s">
-        <v>203</v>
+        <v>219</v>
       </c>
       <c r="D2" s="13" t="s">
-        <v>204</v>
+        <v>220</v>
       </c>
       <c r="F2" s="24"/>
     </row>
@@ -3436,7 +3721,7 @@
       </c>
       <c r="B3" s="4"/>
       <c r="C3" s="3" t="s">
-        <v>205</v>
+        <v>221</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="15.75">
@@ -3444,13 +3729,13 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>206</v>
+        <v>222</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D4" t="s">
-        <v>207</v>
+        <v>223</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="15">
@@ -3458,13 +3743,13 @@
         <v>3</v>
       </c>
       <c r="B5" s="25" t="s">
-        <v>208</v>
+        <v>224</v>
       </c>
       <c r="C5" s="18" t="s">
-        <v>209</v>
+        <v>225</v>
       </c>
       <c r="D5" t="s">
-        <v>210</v>
+        <v>226</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="15">
@@ -3472,13 +3757,13 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>211</v>
+        <v>227</v>
       </c>
       <c r="C6" s="18" t="s">
-        <v>212</v>
+        <v>228</v>
       </c>
       <c r="D6" t="s">
-        <v>213</v>
+        <v>229</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="15.75">
@@ -3486,13 +3771,13 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>214</v>
+        <v>230</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>215</v>
+        <v>231</v>
       </c>
       <c r="D7" t="s">
-        <v>216</v>
+        <v>232</v>
       </c>
     </row>
     <row r="8" spans="1:6">
@@ -3500,13 +3785,13 @@
         <v>1</v>
       </c>
       <c r="B8" s="26" t="s">
-        <v>217</v>
+        <v>233</v>
       </c>
       <c r="C8" s="18" t="s">
-        <v>218</v>
+        <v>234</v>
       </c>
       <c r="D8" t="s">
-        <v>219</v>
+        <v>235</v>
       </c>
     </row>
     <row r="9" spans="1:6">
@@ -3514,13 +3799,13 @@
         <v>2</v>
       </c>
       <c r="B9" s="17" t="s">
-        <v>206</v>
+        <v>222</v>
       </c>
       <c r="C9" s="18" t="s">
-        <v>218</v>
+        <v>234</v>
       </c>
       <c r="D9" t="s">
-        <v>220</v>
+        <v>236</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -3528,10 +3813,10 @@
         <v>3</v>
       </c>
       <c r="B10" s="26" t="s">
-        <v>221</v>
+        <v>237</v>
       </c>
       <c r="C10" s="18" t="s">
-        <v>222</v>
+        <v>238</v>
       </c>
     </row>
     <row r="11" spans="1:6">
@@ -3539,10 +3824,10 @@
         <v>4</v>
       </c>
       <c r="B11" s="26" t="s">
-        <v>223</v>
+        <v>239</v>
       </c>
       <c r="C11" s="18" t="s">
-        <v>224</v>
+        <v>240</v>
       </c>
     </row>
     <row r="12" spans="1:6">
@@ -3550,10 +3835,10 @@
         <v>5</v>
       </c>
       <c r="B12" s="26" t="s">
-        <v>225</v>
+        <v>241</v>
       </c>
       <c r="C12" s="18" t="s">
-        <v>226</v>
+        <v>242</v>
       </c>
     </row>
     <row r="13" spans="1:6">
@@ -3561,10 +3846,10 @@
         <v>6</v>
       </c>
       <c r="B13" s="26" t="s">
-        <v>227</v>
+        <v>243</v>
       </c>
       <c r="C13" s="18" t="s">
-        <v>228</v>
+        <v>244</v>
       </c>
     </row>
     <row r="14" spans="1:6">
@@ -3572,10 +3857,10 @@
         <v>7</v>
       </c>
       <c r="B14" s="26" t="s">
-        <v>229</v>
+        <v>245</v>
       </c>
       <c r="C14" s="18" t="s">
-        <v>230</v>
+        <v>246</v>
       </c>
     </row>
     <row r="15" spans="1:6">
@@ -3583,10 +3868,10 @@
         <v>8</v>
       </c>
       <c r="B15" s="26" t="s">
-        <v>231</v>
+        <v>247</v>
       </c>
       <c r="C15" s="18" t="s">
-        <v>232</v>
+        <v>248</v>
       </c>
     </row>
     <row r="16" spans="1:6">
@@ -3594,10 +3879,10 @@
         <v>9</v>
       </c>
       <c r="B16" s="26" t="s">
-        <v>233</v>
+        <v>249</v>
       </c>
       <c r="C16" s="18" t="s">
-        <v>234</v>
+        <v>250</v>
       </c>
     </row>
     <row r="17" spans="1:3">
@@ -3605,10 +3890,10 @@
         <v>10</v>
       </c>
       <c r="B17" s="26" t="s">
-        <v>235</v>
+        <v>251</v>
       </c>
       <c r="C17" s="18" t="s">
-        <v>236</v>
+        <v>252</v>
       </c>
     </row>
     <row r="18" spans="1:3">
@@ -3657,10 +3942,10 @@
         <v>3</v>
       </c>
       <c r="E1" s="23" t="s">
-        <v>201</v>
+        <v>217</v>
       </c>
       <c r="F1" s="24" t="s">
-        <v>202</v>
+        <v>218</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="15.75">
@@ -3669,10 +3954,10 @@
       </c>
       <c r="B2" s="12"/>
       <c r="C2" s="2" t="s">
-        <v>203</v>
+        <v>219</v>
       </c>
       <c r="D2" s="13" t="s">
-        <v>237</v>
+        <v>253</v>
       </c>
       <c r="F2" s="24"/>
     </row>
@@ -3682,7 +3967,7 @@
       </c>
       <c r="B3" s="4"/>
       <c r="C3" s="3" t="s">
-        <v>205</v>
+        <v>221</v>
       </c>
       <c r="D3" s="14"/>
     </row>
@@ -3691,10 +3976,10 @@
         <v>1</v>
       </c>
       <c r="B4" s="26" t="s">
-        <v>238</v>
+        <v>254</v>
       </c>
       <c r="C4" s="18" t="s">
-        <v>209</v>
+        <v>225</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -3702,11 +3987,11 @@
         <v>2</v>
       </c>
       <c r="B5" s="26" t="s">
-        <v>239</v>
+        <v>255</v>
       </c>
       <c r="C5" s="18"/>
       <c r="D5" t="s">
-        <v>240</v>
+        <v>256</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -3714,13 +3999,13 @@
         <v>3</v>
       </c>
       <c r="B6" s="17" t="s">
-        <v>206</v>
+        <v>222</v>
       </c>
       <c r="C6" s="18" t="s">
-        <v>218</v>
+        <v>234</v>
       </c>
       <c r="D6" t="s">
-        <v>241</v>
+        <v>257</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="15"/>
@@ -3769,10 +4054,10 @@
         <v>3</v>
       </c>
       <c r="E1" s="23" t="s">
-        <v>201</v>
+        <v>217</v>
       </c>
       <c r="F1" s="24" t="s">
-        <v>202</v>
+        <v>218</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="15.75">
@@ -3781,10 +4066,10 @@
       </c>
       <c r="B2" s="12"/>
       <c r="C2" s="2" t="s">
-        <v>203</v>
+        <v>219</v>
       </c>
       <c r="D2" s="13" t="s">
-        <v>242</v>
+        <v>258</v>
       </c>
       <c r="F2" s="24"/>
     </row>
@@ -3794,7 +4079,7 @@
       </c>
       <c r="B3" s="4"/>
       <c r="C3" s="3" t="s">
-        <v>205</v>
+        <v>221</v>
       </c>
       <c r="D3" s="14"/>
     </row>
@@ -3803,13 +4088,13 @@
         <v>1</v>
       </c>
       <c r="B4" s="17" t="s">
-        <v>206</v>
+        <v>222</v>
       </c>
       <c r="C4" t="s">
-        <v>218</v>
+        <v>234</v>
       </c>
       <c r="D4" t="s">
-        <v>243</v>
+        <v>259</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="15">
@@ -3817,13 +4102,13 @@
         <v>2</v>
       </c>
       <c r="B5" t="s">
-        <v>239</v>
+        <v>255</v>
       </c>
       <c r="C5" s="27" t="s">
-        <v>244</v>
+        <v>260</v>
       </c>
       <c r="D5" t="s">
-        <v>245</v>
+        <v>261</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="15">
@@ -3831,13 +4116,13 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>246</v>
+        <v>262</v>
       </c>
       <c r="C6" t="s">
-        <v>247</v>
+        <v>263</v>
       </c>
       <c r="D6" t="s">
-        <v>248</v>
+        <v>264</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -3845,10 +4130,10 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>249</v>
+        <v>265</v>
       </c>
       <c r="D7" t="s">
-        <v>250</v>
+        <v>266</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="15"/>
@@ -3875,17 +4160,12 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{64DA77E0-F1AB-4666-9FA9-D1E469D1B50E}">
-  <dimension ref="A1:A2"/>
+  <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" t="s">
-        <v>251</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1">
-      <c r="A2" t="s">
-        <v>252</v>
+        <v>267</v>
       </c>
     </row>
   </sheetData>
@@ -3918,10 +4198,10 @@
         <v>3</v>
       </c>
       <c r="E1" s="23" t="s">
-        <v>201</v>
+        <v>217</v>
       </c>
       <c r="F1" s="24" t="s">
-        <v>202</v>
+        <v>218</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="15.75">
@@ -3930,10 +4210,10 @@
       </c>
       <c r="B2" s="12"/>
       <c r="C2" s="2" t="s">
-        <v>203</v>
+        <v>219</v>
       </c>
       <c r="D2" s="13" t="s">
-        <v>253</v>
+        <v>268</v>
       </c>
       <c r="F2" s="24"/>
     </row>
@@ -3943,7 +4223,7 @@
       </c>
       <c r="B3" s="4"/>
       <c r="C3" s="3" t="s">
-        <v>205</v>
+        <v>221</v>
       </c>
       <c r="D3" s="14"/>
     </row>
@@ -3952,13 +4232,13 @@
         <v>1</v>
       </c>
       <c r="B4" s="17" t="s">
-        <v>206</v>
+        <v>222</v>
       </c>
       <c r="C4" t="s">
-        <v>218</v>
+        <v>234</v>
       </c>
       <c r="D4" t="s">
-        <v>243</v>
+        <v>259</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -3966,10 +4246,10 @@
         <v>2</v>
       </c>
       <c r="B5" t="s">
-        <v>239</v>
+        <v>255</v>
       </c>
       <c r="D5" t="s">
-        <v>254</v>
+        <v>269</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -3980,7 +4260,7 @@
         <v>2163</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>255</v>
+        <v>270</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -3988,10 +4268,10 @@
         <v>4</v>
       </c>
       <c r="B7" t="s">
-        <v>246</v>
+        <v>262</v>
       </c>
       <c r="C7" t="s">
-        <v>247</v>
+        <v>263</v>
       </c>
     </row>
     <row r="8" spans="1:6">
@@ -3999,46 +4279,46 @@
         <v>5</v>
       </c>
       <c r="B8" t="s">
-        <v>256</v>
+        <v>271</v>
       </c>
       <c r="C8" t="s">
-        <v>247</v>
+        <v>263</v>
       </c>
       <c r="D8" t="s">
-        <v>250</v>
+        <v>266</v>
       </c>
     </row>
     <row r="9" spans="1:6">
       <c r="B9" t="s">
-        <v>257</v>
+        <v>272</v>
       </c>
       <c r="C9" t="s">
-        <v>247</v>
+        <v>263</v>
       </c>
       <c r="D9" t="s">
-        <v>250</v>
+        <v>266</v>
       </c>
     </row>
     <row r="10" spans="1:6">
       <c r="B10" t="s">
-        <v>258</v>
+        <v>273</v>
       </c>
       <c r="C10" t="s">
-        <v>247</v>
+        <v>263</v>
       </c>
       <c r="D10" t="s">
-        <v>250</v>
+        <v>266</v>
       </c>
     </row>
     <row r="11" spans="1:6">
       <c r="B11" t="s">
-        <v>259</v>
+        <v>274</v>
       </c>
       <c r="C11" t="s">
-        <v>247</v>
+        <v>263</v>
       </c>
       <c r="D11" t="s">
-        <v>250</v>
+        <v>266</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="15"/>
@@ -4064,37 +4344,109 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D8FBDE1E-C760-445B-9695-764BC6E6D260}">
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="2" max="2" width="135.140625" customWidth="1"/>
+    <col min="3" max="3" width="9.140625" style="36"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:3">
       <c r="A1" t="s">
-        <v>260</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2">
-      <c r="A2" t="s">
-        <v>261</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="B2" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
       <c r="B3" t="s">
-        <v>262</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
       <c r="B4" t="s">
-        <v>263</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2">
-      <c r="B5" t="s">
-        <v>264</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
+      <c r="A5" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3">
       <c r="A6" t="s">
-        <v>265</v>
+        <v>280</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3">
+      <c r="B7" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3">
+      <c r="B8" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3">
+      <c r="B9" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3">
+      <c r="A10" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3">
+      <c r="B11" s="28" t="s">
+        <v>30</v>
+      </c>
+      <c r="C11" s="40" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3">
+      <c r="B12" s="28" t="s">
+        <v>152</v>
+      </c>
+      <c r="C12" s="40" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3">
+      <c r="B13" s="28" t="s">
+        <v>112</v>
+      </c>
+      <c r="C13" s="40" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3">
+      <c r="B14" s="28" t="s">
+        <v>156</v>
+      </c>
+      <c r="C14" s="40" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3">
+      <c r="B15" s="28" t="s">
+        <v>171</v>
+      </c>
+      <c r="C15" s="40" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3">
+      <c r="B16" t="s">
+        <v>185</v>
+      </c>
+      <c r="C16" s="36" t="s">
+        <v>290</v>
       </c>
     </row>
   </sheetData>
@@ -4118,6 +4470,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101005492B0D1FFC29F46A6C84B04A9E45DCD" ma:contentTypeVersion="22" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="9d86676530458718566c434f3d00fb00">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="6cfc1733-88f5-48e0-9764-36858cbb8ae4" xmlns:ns3="aa93555b-d831-4975-9519-1e883dd949cb" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="48c710b0582ffb978c740d638038b11b" ns1:_="" ns2:_="" ns3:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -4405,25 +4766,16 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9B1B0E3B-34D8-4419-8A30-3BFDCB297D04}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7A0B3543-6925-4BFA-B948-78D0BA20AD89}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{94F315A0-5888-418F-8FBD-82460C37FA32}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{94F315A0-5888-418F-8FBD-82460C37FA32}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7A0B3543-6925-4BFA-B948-78D0BA20AD89}"/>
 </file>
 
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>